<commit_message>
I should adjust the diff
</commit_message>
<xml_diff>
--- a/DataAnalysis/CI/0.05/Results.xlsx
+++ b/DataAnalysis/CI/0.05/Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utente\Desktop\CultureAwarenessTest\DataAnalysis\CI\0.05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B343D2EE-9133-4F32-902A-F5041EE2736F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67EACD23-A803-4453-92A3-24F75265FA3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="81">
   <si>
     <t>Dati originali</t>
   </si>
@@ -344,13 +344,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -1044,72 +1043,34 @@
         <v>20</v>
       </c>
       <c r="G21">
-        <v>15.05</v>
+        <v>18.7</v>
       </c>
       <c r="H21">
-        <v>1.571446608843089</v>
+        <v>2.7748873851023195</v>
       </c>
       <c r="I21">
-        <v>19.8</v>
+        <v>18.5</v>
       </c>
       <c r="J21">
-        <v>2.9925834249951238</v>
+        <v>1.541103500742244</v>
       </c>
       <c r="K21">
-        <v>27.35</v>
+        <v>27.5</v>
       </c>
       <c r="L21">
-        <v>3.1976553910638899</v>
+        <v>1.2247448713915889</v>
       </c>
       <c r="M21">
-        <v>20.733333333333334</v>
+        <v>21.566666666666666</v>
       </c>
       <c r="N21">
-        <v>1.2794674818208691</v>
+        <v>1.4841757907262121</v>
       </c>
       <c r="O21">
-        <v>5.6833333333333327</v>
+        <v>3.9666666666666663</v>
       </c>
       <c r="P21">
-        <v>1.780293359096877</v>
-      </c>
-    </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="D22" t="s">
-        <v>71</v>
-      </c>
-      <c r="F22" t="s">
-        <v>20</v>
-      </c>
-      <c r="G22">
-        <v>15.05</v>
-      </c>
-      <c r="H22">
-        <v>1.571446608843089</v>
-      </c>
-      <c r="I22">
-        <v>19.8</v>
-      </c>
-      <c r="J22">
-        <v>2.9925834249951238</v>
-      </c>
-      <c r="K22">
-        <v>27.35</v>
-      </c>
-      <c r="L22">
-        <v>3.1976553910638899</v>
-      </c>
-      <c r="M22">
-        <v>20.733333333333334</v>
-      </c>
-      <c r="N22">
-        <v>1.2794674818208691</v>
-      </c>
-      <c r="O22">
-        <v>5.6833333333333327</v>
-      </c>
-      <c r="P22">
-        <v>1.780293359096877</v>
+        <v>0.74907350180814036</v>
       </c>
     </row>
     <row r="23" spans="2:16" x14ac:dyDescent="0.3">
@@ -4816,23 +4777,23 @@
         <v>73</v>
       </c>
       <c r="R3">
-        <f t="shared" ref="R3:R34" si="0">AVERAGE(C3:D3)</f>
+        <f t="shared" ref="R3:R11" si="0">AVERAGE(C3:D3)</f>
         <v>15</v>
       </c>
       <c r="S3">
-        <f t="shared" ref="S3:S34" si="1">AVERAGE(H3,I3)</f>
+        <f t="shared" ref="S3:S11" si="1">AVERAGE(H3,I3)</f>
         <v>22</v>
       </c>
       <c r="T3">
-        <f t="shared" ref="T3:T34" si="2">AVERAGE(M3:N3)</f>
+        <f t="shared" ref="T3:T11" si="2">AVERAGE(M3:N3)</f>
         <v>24.5</v>
       </c>
       <c r="U3">
-        <f t="shared" ref="U3:U34" si="3">AVERAGE(R3:T3)</f>
+        <f t="shared" ref="U3:U11" si="3">AVERAGE(R3:T3)</f>
         <v>20.5</v>
       </c>
       <c r="AD3">
-        <f t="shared" ref="AD3:AD34" si="4">MIN(R3:T3)</f>
+        <f t="shared" ref="AD3:AD11" si="4">MIN(R3:T3)</f>
         <v>15</v>
       </c>
       <c r="AE3">
@@ -5411,16 +5372,16 @@
       </c>
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B4" s="3">
+      <c r="B4">
         <v>82</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4">
         <v>18</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4">
         <v>20</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4">
         <v>80</v>
       </c>
       <c r="F4" s="2"/>
@@ -5515,16 +5476,16 @@
       </c>
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B5" s="3">
+      <c r="B5">
         <v>91</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5">
         <v>9</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5">
         <v>20</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5">
         <v>80</v>
       </c>
       <c r="F5" s="2"/>
@@ -5579,16 +5540,16 @@
       </c>
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B6" s="3">
+      <c r="B6">
         <v>82</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6">
         <v>18</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6">
         <v>8</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6">
         <v>92</v>
       </c>
       <c r="F6" s="2"/>
@@ -5643,16 +5604,16 @@
       </c>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B7" s="3">
+      <c r="B7">
         <v>89</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7">
         <v>11</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7">
         <v>18</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7">
         <v>82</v>
       </c>
       <c r="F7" s="2"/>
@@ -5707,16 +5668,16 @@
       </c>
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B8" s="3">
+      <c r="B8">
         <v>84</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8">
         <v>16</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8">
         <v>10</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8">
         <v>90</v>
       </c>
       <c r="F8" s="2"/>
@@ -5771,16 +5732,16 @@
       </c>
     </row>
     <row r="9" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B9" s="3">
+      <c r="B9">
         <v>86</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9">
         <v>14</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9">
         <v>15</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9">
         <v>85</v>
       </c>
       <c r="F9" s="2"/>
@@ -5835,16 +5796,16 @@
       </c>
     </row>
     <row r="10" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B10" s="3">
+      <c r="B10">
         <v>80</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10">
         <v>20</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10">
         <v>11</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E10">
         <v>89</v>
       </c>
       <c r="F10" s="2"/>
@@ -13346,43 +13307,71 @@
         <v>73</v>
       </c>
       <c r="Q16">
-        <f t="shared" ref="Q14:Q23" si="6">AVERAGE(C16:D16)</f>
+        <f t="shared" ref="Q16:Q23" si="6">AVERAGE(C16:D16)</f>
         <v>16.5</v>
       </c>
       <c r="R16">
-        <f t="shared" ref="R14:R23" si="7">AVERAGE(H16:I16)</f>
+        <f t="shared" ref="R16:R23" si="7">AVERAGE(H16:I16)</f>
         <v>22</v>
       </c>
       <c r="S16">
-        <f t="shared" ref="S14:S23" si="8">AVERAGE(M16:N16)</f>
+        <f t="shared" ref="S16:S23" si="8">AVERAGE(M16:N16)</f>
         <v>30</v>
       </c>
       <c r="T16">
-        <f t="shared" ref="T14:T23" si="9">AVERAGE(Q16:S16)</f>
+        <f t="shared" ref="T16:T23" si="9">AVERAGE(Q16:S16)</f>
         <v>22.833333333333332</v>
       </c>
       <c r="U16">
-        <f>AVERAGE(Q16:Q23)</f>
+        <f>AVERAGE(Q16:Q25)</f>
         <v>15.875</v>
       </c>
+      <c r="V16">
+        <f>_xlfn.STDEV.S(Q16:Q25)</f>
+        <v>1.3024701806293193</v>
+      </c>
+      <c r="W16">
+        <f>AVERAGE(R16:R25)</f>
+        <v>19.8125</v>
+      </c>
+      <c r="X16">
+        <f>_xlfn.STDEV.S(R16:R25)</f>
+        <v>2.8652785952802966</v>
+      </c>
+      <c r="Y16">
+        <f>AVERAGE(S16:S25)</f>
+        <v>28.375</v>
+      </c>
+      <c r="Z16">
+        <f>_xlfn.STDEV.S(S16:S25)</f>
+        <v>2.489262656175232</v>
+      </c>
       <c r="AA16">
-        <f>AVERAGE(T16:T23)</f>
+        <f>AVERAGE(T16:T25)</f>
         <v>21.354166666666668</v>
       </c>
+      <c r="AB16">
+        <f>_xlfn.STDEV.S(T16:T25)</f>
+        <v>1.456887037923613</v>
+      </c>
       <c r="AC16">
-        <f t="shared" ref="AC14:AC23" si="10">MIN(Q16:S16)</f>
+        <f t="shared" ref="AC16:AC23" si="10">MIN(Q16:S16)</f>
         <v>16.5</v>
       </c>
       <c r="AD16">
-        <f t="shared" ref="AD14:AD23" si="11">T16-AC16</f>
+        <f t="shared" ref="AD16:AD23" si="11">T16-AC16</f>
         <v>6.3333333333333321</v>
       </c>
       <c r="AE16">
-        <f>AVERAGE(AD16:AD23)</f>
+        <f>AVERAGE(AD16:AD25)</f>
         <v>5.4791666666666661</v>
       </c>
-    </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.3">
+      <c r="AF16">
+        <f>_xlfn.STDEV.S(AD16:AD25)</f>
+        <v>1.7399085453068361</v>
+      </c>
+    </row>
+    <row r="17" spans="1:32" x14ac:dyDescent="0.3">
       <c r="B17">
         <v>88</v>
       </c>
@@ -13444,7 +13433,7 @@
         <v>7.8333333333333321</v>
       </c>
     </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:32" x14ac:dyDescent="0.3">
       <c r="B18">
         <v>85</v>
       </c>
@@ -13506,7 +13495,7 @@
         <v>3.1666666666666679</v>
       </c>
     </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:32" x14ac:dyDescent="0.3">
       <c r="B19">
         <v>90</v>
       </c>
@@ -13568,7 +13557,7 @@
         <v>7.3333333333333321</v>
       </c>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:32" x14ac:dyDescent="0.3">
       <c r="B20">
         <v>88</v>
       </c>
@@ -13630,7 +13619,7 @@
         <v>4.1666666666666679</v>
       </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:32" x14ac:dyDescent="0.3">
       <c r="B21">
         <v>87</v>
       </c>
@@ -13692,7 +13681,7 @@
         <v>6.1666666666666679</v>
       </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:32" x14ac:dyDescent="0.3">
       <c r="B22">
         <v>88</v>
       </c>
@@ -13754,7 +13743,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:32" x14ac:dyDescent="0.3">
       <c r="B23">
         <v>92</v>
       </c>
@@ -13816,17 +13805,17 @@
         <v>5.3333333333333321</v>
       </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="26" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:32" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="27" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:32" x14ac:dyDescent="0.3">
       <c r="B27">
         <v>88</v>
       </c>
@@ -13864,39 +13853,71 @@
         <v>69</v>
       </c>
       <c r="Q27">
-        <f t="shared" ref="Q24:Q31" si="12">AVERAGE(C27:D27)</f>
+        <f t="shared" ref="Q27:Q31" si="12">AVERAGE(C27:D27)</f>
         <v>15.5</v>
       </c>
       <c r="R27">
-        <f t="shared" ref="R24:R31" si="13">AVERAGE(H27:I27)</f>
+        <f t="shared" ref="R27:R31" si="13">AVERAGE(H27:I27)</f>
         <v>17</v>
       </c>
       <c r="S27">
-        <f t="shared" ref="S24:S31" si="14">AVERAGE(M27:N27)</f>
+        <f t="shared" ref="S27:S31" si="14">AVERAGE(M27:N27)</f>
         <v>27.5</v>
       </c>
       <c r="T27">
-        <f t="shared" ref="T24:T31" si="15">AVERAGE(Q27:S27)</f>
+        <f t="shared" ref="T27:T31" si="15">AVERAGE(Q27:S27)</f>
         <v>20</v>
       </c>
+      <c r="U27">
+        <f>AVERAGE(Q27:Q36)</f>
+        <v>18.7</v>
+      </c>
+      <c r="V27">
+        <f>_xlfn.STDEV.S(Q27:Q36)</f>
+        <v>2.7748873851023195</v>
+      </c>
+      <c r="W27">
+        <f>AVERAGE(R27:R36)</f>
+        <v>18.5</v>
+      </c>
+      <c r="X27">
+        <f>_xlfn.STDEV.S(R27:R36)</f>
+        <v>1.541103500742244</v>
+      </c>
+      <c r="Y27">
+        <f>AVERAGE(S27:S36)</f>
+        <v>27.5</v>
+      </c>
+      <c r="Z27">
+        <f>_xlfn.STDEV.S(S27:S36)</f>
+        <v>1.2247448713915889</v>
+      </c>
       <c r="AA27">
-        <f>AVERAGE(T27:T31)</f>
+        <f>AVERAGE(T27:T36)</f>
         <v>21.566666666666666</v>
       </c>
+      <c r="AB27">
+        <f>_xlfn.STDEV.S(T27:T36)</f>
+        <v>1.4841757907262121</v>
+      </c>
       <c r="AC27">
-        <f t="shared" ref="AC24:AC31" si="16">MIN(Q27:S27)</f>
+        <f t="shared" ref="AC27:AC31" si="16">MIN(Q27:S27)</f>
         <v>15.5</v>
       </c>
       <c r="AD27">
-        <f t="shared" ref="AD24:AD31" si="17">T27-AC27</f>
+        <f t="shared" ref="AD27:AD31" si="17">T27-AC27</f>
         <v>4.5</v>
       </c>
       <c r="AE27">
-        <f>AVERAGE(AD27:AD31)</f>
+        <f>AVERAGE(AD27:AD36)</f>
         <v>3.9666666666666663</v>
       </c>
-    </row>
-    <row r="28" spans="1:31" x14ac:dyDescent="0.3">
+      <c r="AF27">
+        <f>_xlfn.STDEV.S(AD27:AD36)</f>
+        <v>0.74907350180814036</v>
+      </c>
+    </row>
+    <row r="28" spans="1:32" x14ac:dyDescent="0.3">
       <c r="B28">
         <v>85</v>
       </c>
@@ -13958,7 +13979,7 @@
         <v>4.3333333333333321</v>
       </c>
     </row>
-    <row r="29" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:32" x14ac:dyDescent="0.3">
       <c r="B29">
         <v>83</v>
       </c>
@@ -14020,7 +14041,7 @@
         <v>4.3333333333333321</v>
       </c>
     </row>
-    <row r="30" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:32" x14ac:dyDescent="0.3">
       <c r="B30">
         <v>88</v>
       </c>
@@ -14082,7 +14103,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:32" x14ac:dyDescent="0.3">
       <c r="B31">
         <v>80</v>
       </c>

</xml_diff>

<commit_message>
DataAnalysis updated for adv
</commit_message>
<xml_diff>
--- a/DataAnalysis/CI/0.05/Results.xlsx
+++ b/DataAnalysis/CI/0.05/Results.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utente\Desktop\CultureAwarenessTest\DataAnalysis\CI\0.05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B46356DC-3BE6-49E9-B246-3E1A1199FC6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFE49676-538D-4FC1-B49D-DF8244159C4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="83">
   <si>
     <t>Dati originali</t>
   </si>
@@ -295,6 +295,12 @@
   </si>
   <si>
     <t>88,12,19,81</t>
+  </si>
+  <si>
+    <t>try3</t>
+  </si>
+  <si>
+    <t>DIFFTry3</t>
   </si>
 </sst>
 </file>
@@ -869,6 +875,41 @@
         <v>0.87589712135373932</v>
       </c>
     </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="C11" t="s">
+        <v>82</v>
+      </c>
+      <c r="G11">
+        <v>17.625</v>
+      </c>
+      <c r="H11">
+        <v>1.796988221070652</v>
+      </c>
+      <c r="I11">
+        <v>21.375</v>
+      </c>
+      <c r="J11">
+        <v>1.8874586088176875</v>
+      </c>
+      <c r="K11">
+        <v>31.375</v>
+      </c>
+      <c r="L11">
+        <v>1.6520189667999174</v>
+      </c>
+      <c r="M11">
+        <v>23.458333333333332</v>
+      </c>
+      <c r="N11">
+        <v>0.49767980186580402</v>
+      </c>
+      <c r="O11">
+        <v>5.833333333333333</v>
+      </c>
+      <c r="P11">
+        <v>1.3402597868683128</v>
+      </c>
+    </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>62</v>
@@ -5304,7 +5345,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F319F6D0-ABAC-48C6-A867-062B0035D0C5}">
-  <dimension ref="A2:AF10"/>
+  <dimension ref="A2:AF15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="2" spans="1:32" x14ac:dyDescent="0.3">
@@ -5857,6 +5898,299 @@
       <c r="V10">
         <f t="shared" si="5"/>
         <v>7.1666666666666679</v>
+      </c>
+    </row>
+    <row r="11" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="12" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B12">
+        <v>82</v>
+      </c>
+      <c r="C12">
+        <v>18</v>
+      </c>
+      <c r="D12">
+        <v>15</v>
+      </c>
+      <c r="E12">
+        <v>85</v>
+      </c>
+      <c r="G12">
+        <v>63</v>
+      </c>
+      <c r="H12">
+        <v>37</v>
+      </c>
+      <c r="I12">
+        <v>9</v>
+      </c>
+      <c r="J12">
+        <v>91</v>
+      </c>
+      <c r="L12">
+        <v>57</v>
+      </c>
+      <c r="M12">
+        <v>43</v>
+      </c>
+      <c r="N12">
+        <v>18</v>
+      </c>
+      <c r="O12">
+        <v>82</v>
+      </c>
+      <c r="Q12">
+        <f t="shared" ref="Q11:Q15" si="6">AVERAGE(C12,D12)</f>
+        <v>16.5</v>
+      </c>
+      <c r="R12">
+        <f t="shared" ref="R11:R15" si="7">AVERAGE(H12,I12)</f>
+        <v>23</v>
+      </c>
+      <c r="S12">
+        <f t="shared" ref="S11:S15" si="8">AVERAGE(M12,N12)</f>
+        <v>30.5</v>
+      </c>
+      <c r="T12">
+        <f t="shared" ref="T11:T15" si="9">AVERAGE(Q12:S12)</f>
+        <v>23.333333333333332</v>
+      </c>
+      <c r="U12">
+        <f t="shared" ref="U11:U15" si="10">MIN(Q12:S12)</f>
+        <v>16.5</v>
+      </c>
+      <c r="V12">
+        <f t="shared" ref="V11:V15" si="11">T12-U12</f>
+        <v>6.8333333333333321</v>
+      </c>
+      <c r="W12">
+        <f>AVERAGE(Q12:Q18)</f>
+        <v>17.625</v>
+      </c>
+      <c r="X12">
+        <f>_xlfn.STDEV.S(Q12:Q18)</f>
+        <v>1.796988221070652</v>
+      </c>
+      <c r="Y12">
+        <f>AVERAGE(R12:R18)</f>
+        <v>21.375</v>
+      </c>
+      <c r="Z12">
+        <f>_xlfn.STDEV.S(R12:R18)</f>
+        <v>1.8874586088176875</v>
+      </c>
+      <c r="AA12">
+        <f>AVERAGE(S12:S18)</f>
+        <v>31.375</v>
+      </c>
+      <c r="AB12">
+        <f>_xlfn.STDEV.S(S12:S18)</f>
+        <v>1.6520189667999174</v>
+      </c>
+      <c r="AC12">
+        <f>AVERAGE(T12:T18)</f>
+        <v>23.458333333333332</v>
+      </c>
+      <c r="AD12">
+        <f>_xlfn.STDEV.S(T12:T18)</f>
+        <v>0.49767980186580402</v>
+      </c>
+      <c r="AE12">
+        <f>AVERAGE(V12:V18)</f>
+        <v>5.833333333333333</v>
+      </c>
+      <c r="AF12">
+        <f>_xlfn.STDEV.S(V12:V18)</f>
+        <v>1.3402597868683128</v>
+      </c>
+    </row>
+    <row r="13" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B13">
+        <v>84</v>
+      </c>
+      <c r="C13">
+        <v>16</v>
+      </c>
+      <c r="D13">
+        <v>16</v>
+      </c>
+      <c r="E13">
+        <v>84</v>
+      </c>
+      <c r="G13">
+        <v>63</v>
+      </c>
+      <c r="H13">
+        <v>37</v>
+      </c>
+      <c r="I13">
+        <v>3</v>
+      </c>
+      <c r="J13">
+        <v>97</v>
+      </c>
+      <c r="L13">
+        <v>56</v>
+      </c>
+      <c r="M13">
+        <v>44</v>
+      </c>
+      <c r="N13">
+        <v>22</v>
+      </c>
+      <c r="O13">
+        <v>78</v>
+      </c>
+      <c r="Q13">
+        <f t="shared" si="6"/>
+        <v>16</v>
+      </c>
+      <c r="R13">
+        <f t="shared" si="7"/>
+        <v>20</v>
+      </c>
+      <c r="S13">
+        <f t="shared" si="8"/>
+        <v>33</v>
+      </c>
+      <c r="T13">
+        <f t="shared" si="9"/>
+        <v>23</v>
+      </c>
+      <c r="U13">
+        <f t="shared" si="10"/>
+        <v>16</v>
+      </c>
+      <c r="V13">
+        <f t="shared" si="11"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B14">
+        <v>82</v>
+      </c>
+      <c r="C14">
+        <v>18</v>
+      </c>
+      <c r="D14">
+        <v>22</v>
+      </c>
+      <c r="E14">
+        <v>78</v>
+      </c>
+      <c r="G14">
+        <v>67</v>
+      </c>
+      <c r="H14">
+        <v>33</v>
+      </c>
+      <c r="I14">
+        <v>13</v>
+      </c>
+      <c r="J14">
+        <v>87</v>
+      </c>
+      <c r="L14">
+        <v>67</v>
+      </c>
+      <c r="M14">
+        <v>33</v>
+      </c>
+      <c r="N14">
+        <v>26</v>
+      </c>
+      <c r="O14">
+        <v>74</v>
+      </c>
+      <c r="Q14">
+        <f t="shared" si="6"/>
+        <v>20</v>
+      </c>
+      <c r="R14">
+        <f t="shared" si="7"/>
+        <v>23</v>
+      </c>
+      <c r="S14">
+        <f t="shared" si="8"/>
+        <v>29.5</v>
+      </c>
+      <c r="T14">
+        <f t="shared" si="9"/>
+        <v>24.166666666666668</v>
+      </c>
+      <c r="U14">
+        <f t="shared" si="10"/>
+        <v>20</v>
+      </c>
+      <c r="V14">
+        <f t="shared" si="11"/>
+        <v>4.1666666666666679</v>
+      </c>
+    </row>
+    <row r="15" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B15">
+        <v>88</v>
+      </c>
+      <c r="C15">
+        <v>12</v>
+      </c>
+      <c r="D15">
+        <v>24</v>
+      </c>
+      <c r="E15">
+        <v>76</v>
+      </c>
+      <c r="G15">
+        <v>67</v>
+      </c>
+      <c r="H15">
+        <v>33</v>
+      </c>
+      <c r="I15">
+        <v>6</v>
+      </c>
+      <c r="J15">
+        <v>94</v>
+      </c>
+      <c r="L15">
+        <v>68</v>
+      </c>
+      <c r="M15">
+        <v>32</v>
+      </c>
+      <c r="N15">
+        <v>33</v>
+      </c>
+      <c r="O15">
+        <v>67</v>
+      </c>
+      <c r="Q15">
+        <f t="shared" si="6"/>
+        <v>18</v>
+      </c>
+      <c r="R15">
+        <f t="shared" si="7"/>
+        <v>19.5</v>
+      </c>
+      <c r="S15">
+        <f t="shared" si="8"/>
+        <v>32.5</v>
+      </c>
+      <c r="T15">
+        <f t="shared" si="9"/>
+        <v>23.333333333333332</v>
+      </c>
+      <c r="U15">
+        <f t="shared" si="10"/>
+        <v>18</v>
+      </c>
+      <c r="V15">
+        <f t="shared" si="11"/>
+        <v>5.3333333333333321</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding data analysis and pulling some results
</commit_message>
<xml_diff>
--- a/DataAnalysis/CI/0.05/Results.xlsx
+++ b/DataAnalysis/CI/0.05/Results.xlsx
@@ -8,28 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utente\Desktop\CultureAwarenessTest\DataAnalysis\CI\0.05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66BA85B2-4747-4CE2-A493-53BBEDD0B5B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFD836C5-5436-4C50-9C59-2E78A5A61823}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
     <sheet name="MIT_DIFF_ONLYMIN_STDAUG" sheetId="19" r:id="rId2"/>
-    <sheet name="MIT_DIFF_ONLYMIN_NOAUG" sheetId="18" r:id="rId3"/>
-    <sheet name="MIT_PARBS_DIFF_ONLYMIN_STDAUG" sheetId="17" r:id="rId4"/>
-    <sheet name="MIT_PARBS_STDAUG" sheetId="14" r:id="rId5"/>
-    <sheet name="MIT_DIFF_STDAUG" sheetId="16" r:id="rId6"/>
-    <sheet name="MIT_DIFF_NOAUG" sheetId="15" r:id="rId7"/>
-    <sheet name="MIT_STDAUG" sheetId="12" r:id="rId8"/>
-    <sheet name="MIT_NOAUG" sheetId="11" r:id="rId9"/>
-    <sheet name="MIT_PARBS_NOAUG" sheetId="13" r:id="rId10"/>
-    <sheet name="STD_IMB_AUG" sheetId="10" r:id="rId11"/>
-    <sheet name="STD_IMB_NOAUG" sheetId="9" r:id="rId12"/>
-    <sheet name="DIFF" sheetId="8" r:id="rId13"/>
-    <sheet name="STD_BAL_ADV_NOCLSDIV" sheetId="7" r:id="rId14"/>
-    <sheet name="STD_BAL_ADV_CLSDIV" sheetId="6" r:id="rId15"/>
-    <sheet name="STD_BAL_STDAUG" sheetId="5" r:id="rId16"/>
-    <sheet name="STD_BAL_NOAUG" sheetId="2" r:id="rId17"/>
+    <sheet name="PARBS_STDAUG" sheetId="20" r:id="rId3"/>
+    <sheet name="MIT_DIFF_ONLYMIN_NOAUG" sheetId="18" r:id="rId4"/>
+    <sheet name="MIT_PARBS_DIFF_ONLYMIN_STDAUG" sheetId="17" r:id="rId5"/>
+    <sheet name="MIT_PARBS_STDAUG" sheetId="14" r:id="rId6"/>
+    <sheet name="MIT_DIFF_STDAUG" sheetId="16" r:id="rId7"/>
+    <sheet name="MIT_DIFF_NOAUG" sheetId="15" r:id="rId8"/>
+    <sheet name="MIT_STDAUG" sheetId="12" r:id="rId9"/>
+    <sheet name="MIT_NOAUG" sheetId="11" r:id="rId10"/>
+    <sheet name="MIT_PARBS_NOAUG" sheetId="13" r:id="rId11"/>
+    <sheet name="STD_IMB_AUG" sheetId="10" r:id="rId12"/>
+    <sheet name="STD_IMB_NOAUG" sheetId="9" r:id="rId13"/>
+    <sheet name="DIFF" sheetId="8" r:id="rId14"/>
+    <sheet name="STD_BAL_ADV_NOCLSDIV" sheetId="7" r:id="rId15"/>
+    <sheet name="STD_BAL_ADV_CLSDIV" sheetId="6" r:id="rId16"/>
+    <sheet name="STD_BAL_STDAUG" sheetId="5" r:id="rId17"/>
+    <sheet name="STD_BAL_NOAUG" sheetId="2" r:id="rId18"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="84">
   <si>
     <t>Dati originali</t>
   </si>
@@ -301,6 +302,9 @@
   </si>
   <si>
     <t>DIFFTry3</t>
+  </si>
+  <si>
+    <t>try</t>
   </si>
 </sst>
 </file>
@@ -636,7 +640,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:P34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.88671875" customWidth="1"/>
@@ -1118,6 +1122,36 @@
       <c r="F22" t="s">
         <v>81</v>
       </c>
+      <c r="G22">
+        <v>16.5</v>
+      </c>
+      <c r="H22">
+        <v>0.70710678118654757</v>
+      </c>
+      <c r="I22">
+        <v>17.25</v>
+      </c>
+      <c r="J22">
+        <v>3.378855822118882</v>
+      </c>
+      <c r="K22">
+        <v>31.25</v>
+      </c>
+      <c r="L22">
+        <v>3.1754264805429417</v>
+      </c>
+      <c r="M22">
+        <v>21.6666666666667</v>
+      </c>
+      <c r="N22">
+        <v>2.2730302828309759</v>
+      </c>
+      <c r="O22">
+        <v>5.7916666666666679</v>
+      </c>
+      <c r="P22">
+        <v>1.6007810593582092</v>
+      </c>
     </row>
     <row r="23" spans="2:16" x14ac:dyDescent="0.3">
       <c r="D23" t="s">
@@ -1159,6 +1193,41 @@
         <v>1.7393858004948073</v>
       </c>
     </row>
+    <row r="25" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="F25" t="s">
+        <v>81</v>
+      </c>
+      <c r="G25">
+        <v>14.875</v>
+      </c>
+      <c r="H25">
+        <v>4.0697051490249265</v>
+      </c>
+      <c r="I25">
+        <v>16.5</v>
+      </c>
+      <c r="J25">
+        <v>2.2730302828309759</v>
+      </c>
+      <c r="K25">
+        <v>27</v>
+      </c>
+      <c r="L25">
+        <v>3.3416562759605704</v>
+      </c>
+      <c r="M25">
+        <v>19.458333333333332</v>
+      </c>
+      <c r="N25">
+        <v>2.1273135553939757</v>
+      </c>
+      <c r="O25">
+        <v>5.2083333333333304</v>
+      </c>
+      <c r="P25">
+        <v>1.674288129546627</v>
+      </c>
+    </row>
     <row r="26" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>72</v>
@@ -1237,49 +1306,122 @@
         <v>0.90215790684828923</v>
       </c>
     </row>
-    <row r="29" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="C29" t="s">
+    <row r="30" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="C30" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="30" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="D30" t="s">
+    <row r="31" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="D31" t="s">
+        <v>71</v>
+      </c>
+      <c r="F31" t="s">
+        <v>81</v>
+      </c>
+      <c r="G31">
+        <v>16</v>
+      </c>
+      <c r="H31">
+        <v>0</v>
+      </c>
+      <c r="I31">
+        <v>15.75</v>
+      </c>
+      <c r="J31">
+        <v>4.5961940777125587</v>
+      </c>
+      <c r="K31">
+        <v>30</v>
+      </c>
+      <c r="L31">
+        <v>3.5355339059327378</v>
+      </c>
+      <c r="M31">
+        <v>20.583333333333332</v>
+      </c>
+      <c r="N31">
+        <v>0.35355339059327379</v>
+      </c>
+      <c r="O31">
+        <v>6.3333333333333321</v>
+      </c>
+      <c r="P31">
+        <v>2.1213203435596459</v>
+      </c>
+    </row>
+    <row r="32" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="D32" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="31" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="E31" t="s">
+    <row r="33" spans="5:16" x14ac:dyDescent="0.3">
+      <c r="E33" t="s">
         <v>71</v>
       </c>
-      <c r="G31">
+      <c r="G33">
         <v>16.375</v>
       </c>
-      <c r="H31">
+      <c r="H33">
         <v>3.3008837200563934</v>
       </c>
-      <c r="I31">
+      <c r="I33">
         <v>20</v>
       </c>
-      <c r="J31">
+      <c r="J33">
         <v>3.3166247903553998</v>
       </c>
-      <c r="K31">
+      <c r="K33">
         <v>26.875</v>
       </c>
-      <c r="L31">
+      <c r="L33">
         <v>1.796988221070652</v>
       </c>
-      <c r="M31">
+      <c r="M33">
         <v>21.083333333333332</v>
       </c>
-      <c r="N31">
+      <c r="N33">
         <v>1.5898986690282424</v>
       </c>
-      <c r="O31">
+      <c r="O33">
         <v>4.708333333333333</v>
       </c>
-      <c r="P31">
+      <c r="P33">
         <v>2.9071272570854019</v>
+      </c>
+    </row>
+    <row r="34" spans="5:16" x14ac:dyDescent="0.3">
+      <c r="F34" t="s">
+        <v>81</v>
+      </c>
+      <c r="G34">
+        <v>14.333333333333334</v>
+      </c>
+      <c r="H34">
+        <v>3.2145502536643153</v>
+      </c>
+      <c r="I34">
+        <v>17.166666666666668</v>
+      </c>
+      <c r="J34">
+        <v>1.2583057392117916</v>
+      </c>
+      <c r="K34">
+        <v>26.6666666666667</v>
+      </c>
+      <c r="L34">
+        <v>4.1633319989322564</v>
+      </c>
+      <c r="M34">
+        <v>19.3888888888889</v>
+      </c>
+      <c r="N34">
+        <v>2.4962935487400935</v>
+      </c>
+      <c r="O34">
+        <v>5.0555555555555562</v>
+      </c>
+      <c r="P34">
+        <v>1.3977495139343468</v>
       </c>
     </row>
   </sheetData>
@@ -1289,6 +1431,557 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8328B926-3ADF-46D7-8F68-CEFFC1D24F6E}">
+  <dimension ref="A2:AF10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="2" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>11</v>
+      </c>
+      <c r="R2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S2" t="s">
+        <v>13</v>
+      </c>
+      <c r="T2" t="s">
+        <v>15</v>
+      </c>
+      <c r="U2" t="s">
+        <v>59</v>
+      </c>
+      <c r="V2" t="s">
+        <v>51</v>
+      </c>
+      <c r="W2" t="s">
+        <v>60</v>
+      </c>
+      <c r="X2" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>14</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>18</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s">
+        <v>70</v>
+      </c>
+      <c r="K3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B4">
+        <v>90</v>
+      </c>
+      <c r="C4">
+        <v>10</v>
+      </c>
+      <c r="D4">
+        <v>15</v>
+      </c>
+      <c r="E4">
+        <v>85</v>
+      </c>
+      <c r="G4">
+        <v>61</v>
+      </c>
+      <c r="H4">
+        <v>39</v>
+      </c>
+      <c r="I4">
+        <v>7</v>
+      </c>
+      <c r="J4">
+        <v>93</v>
+      </c>
+      <c r="L4">
+        <v>72</v>
+      </c>
+      <c r="M4">
+        <v>28</v>
+      </c>
+      <c r="N4">
+        <v>20</v>
+      </c>
+      <c r="O4">
+        <v>80</v>
+      </c>
+      <c r="Q4">
+        <f>AVERAGE(C4,D4)</f>
+        <v>12.5</v>
+      </c>
+      <c r="R4">
+        <f>AVERAGE(H4,I4)</f>
+        <v>23</v>
+      </c>
+      <c r="S4">
+        <f>AVERAGE(M4,N4)</f>
+        <v>24</v>
+      </c>
+      <c r="T4">
+        <f>AVERAGE(Q4:S4)</f>
+        <v>19.833333333333332</v>
+      </c>
+      <c r="U4">
+        <f>AVERAGE(Q4:Q10)</f>
+        <v>14.214285714285714</v>
+      </c>
+      <c r="V4">
+        <f>_xlfn.STDEV.S(Q4:Q10)</f>
+        <v>2.0987524639084736</v>
+      </c>
+      <c r="W4">
+        <f>AVERAGE(R4:R10)</f>
+        <v>23</v>
+      </c>
+      <c r="X4">
+        <f>_xlfn.STDEV.S(R4:R10)</f>
+        <v>2.5495097567963922</v>
+      </c>
+      <c r="Y4">
+        <f>AVERAGE(S4:S10)</f>
+        <v>31.428571428571427</v>
+      </c>
+      <c r="Z4">
+        <f>_xlfn.STDEV.S(S4:S10)</f>
+        <v>5.2870011303555522</v>
+      </c>
+      <c r="AA4">
+        <f>AVERAGE(T4:T10)</f>
+        <v>22.88095238095238</v>
+      </c>
+      <c r="AB4">
+        <f>_xlfn.STDEV.S(T4:T10)</f>
+        <v>2.2601914981845255</v>
+      </c>
+      <c r="AC4">
+        <f>MIN(Q4:S4)</f>
+        <v>12.5</v>
+      </c>
+      <c r="AD4">
+        <f>T4-AC4</f>
+        <v>7.3333333333333321</v>
+      </c>
+      <c r="AE4">
+        <f>AVERAGE(AD4:AD10)</f>
+        <v>8.6666666666666661</v>
+      </c>
+      <c r="AF4">
+        <f>_xlfn.STDEV.S(AD4:AD10)</f>
+        <v>2.0971762320196583</v>
+      </c>
+    </row>
+    <row r="5" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B5">
+        <v>87</v>
+      </c>
+      <c r="C5">
+        <v>13</v>
+      </c>
+      <c r="D5">
+        <v>15</v>
+      </c>
+      <c r="E5">
+        <v>85</v>
+      </c>
+      <c r="G5">
+        <v>49</v>
+      </c>
+      <c r="H5">
+        <v>51</v>
+      </c>
+      <c r="I5">
+        <v>2</v>
+      </c>
+      <c r="J5">
+        <v>98</v>
+      </c>
+      <c r="L5">
+        <v>58</v>
+      </c>
+      <c r="M5">
+        <v>42</v>
+      </c>
+      <c r="N5">
+        <v>25</v>
+      </c>
+      <c r="O5">
+        <v>75</v>
+      </c>
+      <c r="Q5">
+        <f t="shared" ref="Q5:Q10" si="0">AVERAGE(C5,D5)</f>
+        <v>14</v>
+      </c>
+      <c r="R5">
+        <f t="shared" ref="R5:R10" si="1">AVERAGE(H5,I5)</f>
+        <v>26.5</v>
+      </c>
+      <c r="S5">
+        <f t="shared" ref="S5:S10" si="2">AVERAGE(M5,N5)</f>
+        <v>33.5</v>
+      </c>
+      <c r="T5">
+        <f t="shared" ref="T5:T10" si="3">AVERAGE(Q5:S5)</f>
+        <v>24.666666666666668</v>
+      </c>
+      <c r="AC5">
+        <f t="shared" ref="AC5:AC10" si="4">MIN(Q5:S5)</f>
+        <v>14</v>
+      </c>
+      <c r="AD5">
+        <f t="shared" ref="AD5:AD10" si="5">T5-AC5</f>
+        <v>10.666666666666668</v>
+      </c>
+    </row>
+    <row r="6" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6">
+        <v>84</v>
+      </c>
+      <c r="C6">
+        <v>16</v>
+      </c>
+      <c r="D6">
+        <v>19</v>
+      </c>
+      <c r="E6">
+        <v>81</v>
+      </c>
+      <c r="G6">
+        <v>56</v>
+      </c>
+      <c r="H6">
+        <v>44</v>
+      </c>
+      <c r="I6">
+        <v>8</v>
+      </c>
+      <c r="J6">
+        <v>92</v>
+      </c>
+      <c r="L6">
+        <v>69</v>
+      </c>
+      <c r="M6">
+        <v>31</v>
+      </c>
+      <c r="N6">
+        <v>25</v>
+      </c>
+      <c r="O6">
+        <v>75</v>
+      </c>
+      <c r="Q6">
+        <f t="shared" si="0"/>
+        <v>17.5</v>
+      </c>
+      <c r="R6">
+        <f t="shared" si="1"/>
+        <v>26</v>
+      </c>
+      <c r="S6">
+        <f t="shared" si="2"/>
+        <v>28</v>
+      </c>
+      <c r="T6">
+        <f t="shared" si="3"/>
+        <v>23.833333333333332</v>
+      </c>
+      <c r="AC6">
+        <f t="shared" si="4"/>
+        <v>17.5</v>
+      </c>
+      <c r="AD6">
+        <f t="shared" si="5"/>
+        <v>6.3333333333333321</v>
+      </c>
+    </row>
+    <row r="7" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B7">
+        <v>90</v>
+      </c>
+      <c r="C7">
+        <v>10</v>
+      </c>
+      <c r="D7">
+        <v>12</v>
+      </c>
+      <c r="E7">
+        <v>88</v>
+      </c>
+      <c r="G7">
+        <v>67</v>
+      </c>
+      <c r="H7">
+        <v>33</v>
+      </c>
+      <c r="I7">
+        <v>8</v>
+      </c>
+      <c r="J7">
+        <v>92</v>
+      </c>
+      <c r="L7">
+        <v>58</v>
+      </c>
+      <c r="M7">
+        <v>42</v>
+      </c>
+      <c r="N7">
+        <v>23</v>
+      </c>
+      <c r="O7">
+        <v>77</v>
+      </c>
+      <c r="Q7">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="R7">
+        <f t="shared" si="1"/>
+        <v>20.5</v>
+      </c>
+      <c r="S7">
+        <f t="shared" si="2"/>
+        <v>32.5</v>
+      </c>
+      <c r="T7">
+        <f t="shared" si="3"/>
+        <v>21.333333333333332</v>
+      </c>
+      <c r="AC7">
+        <f t="shared" si="4"/>
+        <v>11</v>
+      </c>
+      <c r="AD7">
+        <f t="shared" si="5"/>
+        <v>10.333333333333332</v>
+      </c>
+    </row>
+    <row r="8" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B8">
+        <v>89</v>
+      </c>
+      <c r="C8">
+        <v>11</v>
+      </c>
+      <c r="D8">
+        <v>19</v>
+      </c>
+      <c r="E8">
+        <v>81</v>
+      </c>
+      <c r="G8">
+        <v>62</v>
+      </c>
+      <c r="H8">
+        <v>38</v>
+      </c>
+      <c r="I8">
+        <v>9</v>
+      </c>
+      <c r="J8">
+        <v>91</v>
+      </c>
+      <c r="L8">
+        <v>52</v>
+      </c>
+      <c r="M8">
+        <v>48</v>
+      </c>
+      <c r="N8">
+        <v>34</v>
+      </c>
+      <c r="O8">
+        <v>66</v>
+      </c>
+      <c r="Q8">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="R8">
+        <f t="shared" si="1"/>
+        <v>23.5</v>
+      </c>
+      <c r="S8">
+        <f t="shared" si="2"/>
+        <v>41</v>
+      </c>
+      <c r="T8">
+        <f t="shared" si="3"/>
+        <v>26.5</v>
+      </c>
+      <c r="AC8">
+        <f t="shared" si="4"/>
+        <v>15</v>
+      </c>
+      <c r="AD8">
+        <f t="shared" si="5"/>
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B9">
+        <v>88</v>
+      </c>
+      <c r="C9">
+        <v>12</v>
+      </c>
+      <c r="D9">
+        <v>16</v>
+      </c>
+      <c r="E9">
+        <v>84</v>
+      </c>
+      <c r="G9">
+        <v>65</v>
+      </c>
+      <c r="H9">
+        <v>35</v>
+      </c>
+      <c r="I9">
+        <v>8</v>
+      </c>
+      <c r="J9">
+        <v>92</v>
+      </c>
+      <c r="L9">
+        <v>65</v>
+      </c>
+      <c r="M9">
+        <v>35</v>
+      </c>
+      <c r="N9">
+        <v>24</v>
+      </c>
+      <c r="O9">
+        <v>76</v>
+      </c>
+      <c r="Q9">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="R9">
+        <f t="shared" si="1"/>
+        <v>21.5</v>
+      </c>
+      <c r="S9">
+        <f t="shared" si="2"/>
+        <v>29.5</v>
+      </c>
+      <c r="T9">
+        <f t="shared" si="3"/>
+        <v>21.666666666666668</v>
+      </c>
+      <c r="AC9">
+        <f t="shared" si="4"/>
+        <v>14</v>
+      </c>
+      <c r="AD9">
+        <f t="shared" si="5"/>
+        <v>7.6666666666666679</v>
+      </c>
+    </row>
+    <row r="10" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B10">
+        <v>83</v>
+      </c>
+      <c r="C10">
+        <v>17</v>
+      </c>
+      <c r="D10">
+        <v>14</v>
+      </c>
+      <c r="E10">
+        <v>86</v>
+      </c>
+      <c r="G10">
+        <v>64</v>
+      </c>
+      <c r="H10">
+        <v>36</v>
+      </c>
+      <c r="I10">
+        <v>4</v>
+      </c>
+      <c r="J10">
+        <v>96</v>
+      </c>
+      <c r="L10">
+        <v>64</v>
+      </c>
+      <c r="M10">
+        <v>36</v>
+      </c>
+      <c r="N10">
+        <v>27</v>
+      </c>
+      <c r="O10">
+        <v>73</v>
+      </c>
+      <c r="Q10">
+        <f t="shared" si="0"/>
+        <v>15.5</v>
+      </c>
+      <c r="R10">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="S10">
+        <f t="shared" si="2"/>
+        <v>31.5</v>
+      </c>
+      <c r="T10">
+        <f t="shared" si="3"/>
+        <v>22.333333333333332</v>
+      </c>
+      <c r="AC10">
+        <f t="shared" si="4"/>
+        <v>15.5</v>
+      </c>
+      <c r="AD10">
+        <f t="shared" si="5"/>
+        <v>6.8333333333333321</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEC9CF4A-6F3D-4BA0-B506-17E3C93FB04B}">
   <dimension ref="A2:AF9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1777,7 +2470,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84CA6F53-9387-444E-890F-DCD3D83EC80C}">
   <dimension ref="A1:AO99"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4616,7 +5309,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C39A647-64D8-47BC-AD52-3FB80D45AD9F}">
   <dimension ref="A1:AG11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -5348,7 +6041,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F319F6D0-ABAC-48C6-A867-062B0035D0C5}">
   <dimension ref="A2:AF15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -6203,7 +6896,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76F82D8A-1A23-4CF3-9872-DA5B576CDAF9}">
   <dimension ref="A1:AN41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -7640,7 +8333,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8214124B-224B-4F9B-B528-181D112DB9C5}">
   <dimension ref="A1:AL41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -8717,7 +9410,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03D9506E-E2C3-4105-A101-2ED902EAE848}">
   <dimension ref="A1:AR109"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -11253,7 +11946,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D80BAE23-A740-4698-B840-F018E78CD098}">
   <dimension ref="A1:AF5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -11553,7 +12246,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D0CE18A-8B26-4E93-B497-B59E55EFEC0E}">
-  <dimension ref="A2:AF7"/>
+  <dimension ref="A2:AF13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="2" spans="1:32" x14ac:dyDescent="0.3">
@@ -11909,6 +12602,299 @@
       <c r="AD7">
         <f t="shared" si="5"/>
         <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="10" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B10">
+        <v>84</v>
+      </c>
+      <c r="C10">
+        <v>16</v>
+      </c>
+      <c r="D10">
+        <v>11</v>
+      </c>
+      <c r="E10">
+        <v>89</v>
+      </c>
+      <c r="G10">
+        <v>76</v>
+      </c>
+      <c r="H10">
+        <v>24</v>
+      </c>
+      <c r="I10">
+        <v>6</v>
+      </c>
+      <c r="J10">
+        <v>94</v>
+      </c>
+      <c r="L10">
+        <v>67</v>
+      </c>
+      <c r="M10">
+        <v>33</v>
+      </c>
+      <c r="N10">
+        <v>27</v>
+      </c>
+      <c r="O10">
+        <v>73</v>
+      </c>
+      <c r="Q10">
+        <f t="shared" ref="Q10:Q13" si="6">AVERAGE(C10:D10)</f>
+        <v>13.5</v>
+      </c>
+      <c r="R10">
+        <f t="shared" ref="R10:R13" si="7">AVERAGE(H10:I10)</f>
+        <v>15</v>
+      </c>
+      <c r="S10">
+        <f t="shared" ref="S10:S13" si="8">AVERAGE(M10:N10)</f>
+        <v>30</v>
+      </c>
+      <c r="T10">
+        <f t="shared" ref="T10:T13" si="9">AVERAGE(Q10:S10)</f>
+        <v>19.5</v>
+      </c>
+      <c r="U10">
+        <f>AVERAGE(Q10:Q13)</f>
+        <v>14.875</v>
+      </c>
+      <c r="V10">
+        <f>_xlfn.STDEV.S(Q10:Q13)</f>
+        <v>4.0697051490249265</v>
+      </c>
+      <c r="W10">
+        <f>AVERAGE(R10:R13)</f>
+        <v>16.5</v>
+      </c>
+      <c r="X10">
+        <f>_xlfn.STDEV.S(R10:R13)</f>
+        <v>2.2730302828309759</v>
+      </c>
+      <c r="Y10">
+        <f>AVERAGE(S10:S13)</f>
+        <v>27</v>
+      </c>
+      <c r="Z10">
+        <f>_xlfn.STDEV.S(S10:S13)</f>
+        <v>3.3416562759605704</v>
+      </c>
+      <c r="AA10">
+        <f>AVERAGE(T10:T13)</f>
+        <v>19.458333333333332</v>
+      </c>
+      <c r="AB10">
+        <f>_xlfn.STDEV.S(T10:T13)</f>
+        <v>2.1273135553939757</v>
+      </c>
+      <c r="AC10">
+        <f t="shared" ref="AC10:AC13" si="10">MIN(Q10:S10)</f>
+        <v>13.5</v>
+      </c>
+      <c r="AD10">
+        <f t="shared" ref="AD10:AD13" si="11">T10-AC10</f>
+        <v>6</v>
+      </c>
+      <c r="AE10">
+        <f>AVERAGE(AD10:AD13)</f>
+        <v>5.208333333333333</v>
+      </c>
+      <c r="AF10">
+        <f>_xlfn.STDEV.S(AD10:AD13)</f>
+        <v>1.674288129546627</v>
+      </c>
+    </row>
+    <row r="11" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B11">
+        <v>87</v>
+      </c>
+      <c r="C11">
+        <v>13</v>
+      </c>
+      <c r="D11">
+        <v>20</v>
+      </c>
+      <c r="E11">
+        <v>80</v>
+      </c>
+      <c r="G11">
+        <v>78</v>
+      </c>
+      <c r="H11">
+        <v>22</v>
+      </c>
+      <c r="I11">
+        <v>17</v>
+      </c>
+      <c r="J11">
+        <v>83</v>
+      </c>
+      <c r="L11">
+        <v>70</v>
+      </c>
+      <c r="M11">
+        <v>30</v>
+      </c>
+      <c r="N11">
+        <v>29</v>
+      </c>
+      <c r="O11">
+        <v>71</v>
+      </c>
+      <c r="Q11">
+        <f t="shared" si="6"/>
+        <v>16.5</v>
+      </c>
+      <c r="R11">
+        <f t="shared" si="7"/>
+        <v>19.5</v>
+      </c>
+      <c r="S11">
+        <f t="shared" si="8"/>
+        <v>29.5</v>
+      </c>
+      <c r="T11">
+        <f t="shared" si="9"/>
+        <v>21.833333333333332</v>
+      </c>
+      <c r="AC11">
+        <f t="shared" si="10"/>
+        <v>16.5</v>
+      </c>
+      <c r="AD11">
+        <f t="shared" si="11"/>
+        <v>5.3333333333333321</v>
+      </c>
+    </row>
+    <row r="12" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B12">
+        <v>83</v>
+      </c>
+      <c r="C12">
+        <v>17</v>
+      </c>
+      <c r="D12">
+        <v>22</v>
+      </c>
+      <c r="E12">
+        <v>78</v>
+      </c>
+      <c r="G12">
+        <v>74</v>
+      </c>
+      <c r="H12">
+        <v>26</v>
+      </c>
+      <c r="I12">
+        <v>8</v>
+      </c>
+      <c r="J12">
+        <v>92</v>
+      </c>
+      <c r="L12">
+        <v>72</v>
+      </c>
+      <c r="M12">
+        <v>28</v>
+      </c>
+      <c r="N12">
+        <v>18</v>
+      </c>
+      <c r="O12">
+        <v>82</v>
+      </c>
+      <c r="Q12">
+        <f t="shared" si="6"/>
+        <v>19.5</v>
+      </c>
+      <c r="R12">
+        <f t="shared" si="7"/>
+        <v>17</v>
+      </c>
+      <c r="S12">
+        <f t="shared" si="8"/>
+        <v>23</v>
+      </c>
+      <c r="T12">
+        <f t="shared" si="9"/>
+        <v>19.833333333333332</v>
+      </c>
+      <c r="AC12">
+        <f t="shared" si="10"/>
+        <v>17</v>
+      </c>
+      <c r="AD12">
+        <f t="shared" si="11"/>
+        <v>2.8333333333333321</v>
+      </c>
+    </row>
+    <row r="13" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B13">
+        <v>92</v>
+      </c>
+      <c r="C13">
+        <v>8</v>
+      </c>
+      <c r="D13">
+        <v>12</v>
+      </c>
+      <c r="E13">
+        <v>88</v>
+      </c>
+      <c r="G13">
+        <v>79</v>
+      </c>
+      <c r="H13">
+        <v>21</v>
+      </c>
+      <c r="I13">
+        <v>8</v>
+      </c>
+      <c r="J13">
+        <v>92</v>
+      </c>
+      <c r="L13">
+        <v>72</v>
+      </c>
+      <c r="M13">
+        <v>28</v>
+      </c>
+      <c r="N13">
+        <v>23</v>
+      </c>
+      <c r="O13">
+        <v>77</v>
+      </c>
+      <c r="Q13">
+        <f t="shared" si="6"/>
+        <v>10</v>
+      </c>
+      <c r="R13">
+        <f t="shared" si="7"/>
+        <v>14.5</v>
+      </c>
+      <c r="S13">
+        <f t="shared" si="8"/>
+        <v>25.5</v>
+      </c>
+      <c r="T13">
+        <f t="shared" si="9"/>
+        <v>16.666666666666668</v>
+      </c>
+      <c r="AC13">
+        <f t="shared" si="10"/>
+        <v>10</v>
+      </c>
+      <c r="AD13">
+        <f t="shared" si="11"/>
+        <v>6.6666666666666679</v>
       </c>
     </row>
   </sheetData>
@@ -11917,6 +12903,230 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1341680-B8DF-484F-AD8E-90C5FE6FD057}">
+  <dimension ref="B1:AF3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="2:32" x14ac:dyDescent="0.3">
+      <c r="Q1" t="s">
+        <v>11</v>
+      </c>
+      <c r="R1" t="s">
+        <v>12</v>
+      </c>
+      <c r="S1" t="s">
+        <v>13</v>
+      </c>
+      <c r="T1" t="s">
+        <v>15</v>
+      </c>
+      <c r="U1" t="s">
+        <v>59</v>
+      </c>
+      <c r="V1" t="s">
+        <v>51</v>
+      </c>
+      <c r="W1" t="s">
+        <v>60</v>
+      </c>
+      <c r="X1" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>53</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>14</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>18</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="2:32" x14ac:dyDescent="0.3">
+      <c r="B2">
+        <v>81</v>
+      </c>
+      <c r="C2">
+        <v>19</v>
+      </c>
+      <c r="D2">
+        <v>13</v>
+      </c>
+      <c r="E2">
+        <v>87</v>
+      </c>
+      <c r="G2">
+        <v>78</v>
+      </c>
+      <c r="H2">
+        <v>22</v>
+      </c>
+      <c r="I2">
+        <v>3</v>
+      </c>
+      <c r="J2">
+        <v>97</v>
+      </c>
+      <c r="L2">
+        <v>65</v>
+      </c>
+      <c r="M2">
+        <v>35</v>
+      </c>
+      <c r="N2">
+        <v>30</v>
+      </c>
+      <c r="O2">
+        <v>70</v>
+      </c>
+      <c r="Q2">
+        <f>AVERAGE(C2,D2)</f>
+        <v>16</v>
+      </c>
+      <c r="R2">
+        <f>AVERAGE(H2,I2)</f>
+        <v>12.5</v>
+      </c>
+      <c r="S2">
+        <f>AVERAGE(M2,N2)</f>
+        <v>32.5</v>
+      </c>
+      <c r="T2">
+        <f>AVERAGE(Q2:S2)</f>
+        <v>20.333333333333332</v>
+      </c>
+      <c r="U2">
+        <f>AVERAGE(Q2,Q3)</f>
+        <v>16</v>
+      </c>
+      <c r="V2">
+        <f>_xlfn.STDEV.S(Q2,Q3)</f>
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <f>AVERAGE(R2,R3)</f>
+        <v>15.75</v>
+      </c>
+      <c r="X2">
+        <f>_xlfn.STDEV.S(R2,R3)</f>
+        <v>4.5961940777125587</v>
+      </c>
+      <c r="Y2">
+        <f>AVERAGE(S2,S3)</f>
+        <v>30</v>
+      </c>
+      <c r="Z2">
+        <f>_xlfn.STDEV.S(S2,S3)</f>
+        <v>3.5355339059327378</v>
+      </c>
+      <c r="AA2">
+        <f>AVERAGE(T2,T3)</f>
+        <v>20.583333333333332</v>
+      </c>
+      <c r="AB2">
+        <f>_xlfn.STDEV.S(T2,T3)</f>
+        <v>0.35355339059327379</v>
+      </c>
+      <c r="AC2">
+        <f>MIN(Q2:S2)</f>
+        <v>12.5</v>
+      </c>
+      <c r="AD2">
+        <f>(T2-AC2)</f>
+        <v>7.8333333333333321</v>
+      </c>
+      <c r="AE2">
+        <f>AVERAGE(AD2,AD3)</f>
+        <v>6.3333333333333321</v>
+      </c>
+      <c r="AF2">
+        <f>_xlfn.STDEV.S(AD2,AD3)</f>
+        <v>2.1213203435596459</v>
+      </c>
+    </row>
+    <row r="3" spans="2:32" x14ac:dyDescent="0.3">
+      <c r="B3">
+        <v>88</v>
+      </c>
+      <c r="C3">
+        <v>12</v>
+      </c>
+      <c r="D3">
+        <v>20</v>
+      </c>
+      <c r="E3">
+        <v>80</v>
+      </c>
+      <c r="G3">
+        <v>80</v>
+      </c>
+      <c r="H3">
+        <v>20</v>
+      </c>
+      <c r="I3">
+        <v>18</v>
+      </c>
+      <c r="J3">
+        <v>82</v>
+      </c>
+      <c r="L3">
+        <v>72</v>
+      </c>
+      <c r="M3">
+        <v>28</v>
+      </c>
+      <c r="N3">
+        <v>27</v>
+      </c>
+      <c r="O3">
+        <v>73</v>
+      </c>
+      <c r="Q3">
+        <f>AVERAGE(C3,D3)</f>
+        <v>16</v>
+      </c>
+      <c r="R3">
+        <f>AVERAGE(H3,I3)</f>
+        <v>19</v>
+      </c>
+      <c r="S3">
+        <f>AVERAGE(M3,N3)</f>
+        <v>27.5</v>
+      </c>
+      <c r="T3">
+        <f>AVERAGE(Q3:S3)</f>
+        <v>20.833333333333332</v>
+      </c>
+      <c r="AC3">
+        <f>MIN(Q3:S3)</f>
+        <v>16</v>
+      </c>
+      <c r="AD3">
+        <f>(T3-AC3)</f>
+        <v>4.8333333333333321</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E557A7D-364E-47EE-A0F3-0D888512E587}">
   <dimension ref="A2:AF5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -12082,9 +13292,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1B67D71-588A-4985-8ACA-35F7A9B1AF58}">
-  <dimension ref="A2:AF7"/>
+  <dimension ref="A2:AF12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="2" spans="1:32" x14ac:dyDescent="0.3">
@@ -12442,12 +13652,243 @@
         <v>3</v>
       </c>
     </row>
+    <row r="9" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="10" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B10">
+        <v>94</v>
+      </c>
+      <c r="C10">
+        <v>6</v>
+      </c>
+      <c r="D10">
+        <v>18</v>
+      </c>
+      <c r="E10">
+        <v>82</v>
+      </c>
+      <c r="G10">
+        <v>79</v>
+      </c>
+      <c r="H10">
+        <v>21</v>
+      </c>
+      <c r="I10">
+        <v>11</v>
+      </c>
+      <c r="J10">
+        <v>89</v>
+      </c>
+      <c r="L10">
+        <v>60</v>
+      </c>
+      <c r="M10">
+        <v>40</v>
+      </c>
+      <c r="N10">
+        <v>16</v>
+      </c>
+      <c r="O10">
+        <v>84</v>
+      </c>
+      <c r="Q10">
+        <f t="shared" ref="Q10:Q12" si="6">AVERAGE(C10:D10)</f>
+        <v>12</v>
+      </c>
+      <c r="R10">
+        <f t="shared" ref="R10:R12" si="7">AVERAGE(H10:I10)</f>
+        <v>16</v>
+      </c>
+      <c r="S10">
+        <f t="shared" ref="S10:S12" si="8">AVERAGE(M10:N10)</f>
+        <v>28</v>
+      </c>
+      <c r="T10">
+        <f t="shared" ref="T10:T12" si="9">AVERAGE(Q10:S10)</f>
+        <v>18.666666666666668</v>
+      </c>
+      <c r="U10">
+        <f>AVERAGE(Q10:Q13)</f>
+        <v>14.333333333333334</v>
+      </c>
+      <c r="V10">
+        <f>_xlfn.STDEV.S(Q10:Q13)</f>
+        <v>3.2145502536643153</v>
+      </c>
+      <c r="W10">
+        <f>AVERAGE(R10:R13)</f>
+        <v>17.166666666666668</v>
+      </c>
+      <c r="X10">
+        <f>_xlfn.STDEV.S(R10:R13)</f>
+        <v>1.2583057392117916</v>
+      </c>
+      <c r="Y10">
+        <f>AVERAGE(S10:S13)</f>
+        <v>26.666666666666668</v>
+      </c>
+      <c r="Z10">
+        <f>_xlfn.STDEV.S(S10:S13)</f>
+        <v>4.1633319989322564</v>
+      </c>
+      <c r="AA10">
+        <f>AVERAGE(T10:T13)</f>
+        <v>19.388888888888889</v>
+      </c>
+      <c r="AB10">
+        <f>_xlfn.STDEV.S(T10:T13)</f>
+        <v>2.4962935487400935</v>
+      </c>
+      <c r="AC10">
+        <f t="shared" ref="AC10:AC12" si="10">MIN(Q10:S10)</f>
+        <v>12</v>
+      </c>
+      <c r="AD10">
+        <f t="shared" ref="AD10:AD12" si="11">T10-AC10</f>
+        <v>6.6666666666666679</v>
+      </c>
+      <c r="AE10">
+        <f>AVERAGE(AD10:AD13)</f>
+        <v>5.0555555555555562</v>
+      </c>
+      <c r="AF10">
+        <f>_xlfn.STDEV.S(AD10:AD13)</f>
+        <v>1.3977495139343468</v>
+      </c>
+    </row>
+    <row r="11" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B11">
+        <v>86</v>
+      </c>
+      <c r="C11">
+        <v>14</v>
+      </c>
+      <c r="D11">
+        <v>22</v>
+      </c>
+      <c r="E11">
+        <v>78</v>
+      </c>
+      <c r="G11">
+        <v>81</v>
+      </c>
+      <c r="H11">
+        <v>19</v>
+      </c>
+      <c r="I11">
+        <v>18</v>
+      </c>
+      <c r="J11">
+        <v>82</v>
+      </c>
+      <c r="L11">
+        <v>78</v>
+      </c>
+      <c r="M11">
+        <v>22</v>
+      </c>
+      <c r="N11">
+        <v>38</v>
+      </c>
+      <c r="O11">
+        <v>62</v>
+      </c>
+      <c r="Q11">
+        <f t="shared" si="6"/>
+        <v>18</v>
+      </c>
+      <c r="R11">
+        <f t="shared" si="7"/>
+        <v>18.5</v>
+      </c>
+      <c r="S11">
+        <f t="shared" si="8"/>
+        <v>30</v>
+      </c>
+      <c r="T11">
+        <f t="shared" si="9"/>
+        <v>22.166666666666668</v>
+      </c>
+      <c r="AC11">
+        <f t="shared" si="10"/>
+        <v>18</v>
+      </c>
+      <c r="AD11">
+        <f t="shared" si="11"/>
+        <v>4.1666666666666679</v>
+      </c>
+    </row>
+    <row r="12" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B12">
+        <v>91</v>
+      </c>
+      <c r="C12">
+        <v>9</v>
+      </c>
+      <c r="D12">
+        <v>17</v>
+      </c>
+      <c r="E12">
+        <v>83</v>
+      </c>
+      <c r="G12">
+        <v>79</v>
+      </c>
+      <c r="H12">
+        <v>21</v>
+      </c>
+      <c r="I12">
+        <v>13</v>
+      </c>
+      <c r="J12">
+        <v>87</v>
+      </c>
+      <c r="L12">
+        <v>74</v>
+      </c>
+      <c r="M12">
+        <v>26</v>
+      </c>
+      <c r="N12">
+        <v>18</v>
+      </c>
+      <c r="O12">
+        <v>82</v>
+      </c>
+      <c r="Q12">
+        <f t="shared" si="6"/>
+        <v>13</v>
+      </c>
+      <c r="R12">
+        <f t="shared" si="7"/>
+        <v>17</v>
+      </c>
+      <c r="S12">
+        <f t="shared" si="8"/>
+        <v>22</v>
+      </c>
+      <c r="T12">
+        <f t="shared" si="9"/>
+        <v>17.333333333333332</v>
+      </c>
+      <c r="AC12">
+        <f t="shared" si="10"/>
+        <v>13</v>
+      </c>
+      <c r="AD12">
+        <f t="shared" si="11"/>
+        <v>4.3333333333333321</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A366D673-4552-407C-AD95-3B60150A1024}">
   <dimension ref="A2:AF8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -12871,7 +14312,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A4C68C5-0EAB-4233-98F5-D346BC512EB4}">
   <dimension ref="A2:AF31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -14509,7 +15950,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0843B137-6F6F-47C7-80DB-2FF2B4BCD957}">
   <dimension ref="A2:AF5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -14672,9 +16113,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25FCA91D-5E11-4BE7-9F8B-616A902FA88F}">
-  <dimension ref="A2:AF10"/>
+  <dimension ref="A2:AF14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="2" spans="1:32" x14ac:dyDescent="0.3">
@@ -15158,555 +16599,292 @@
         <v>81</v>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8328B926-3ADF-46D7-8F68-CEFFC1D24F6E}">
-  <dimension ref="A2:AF10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q2" t="s">
+    <row r="11" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B11">
+        <v>86</v>
+      </c>
+      <c r="C11">
+        <v>14</v>
+      </c>
+      <c r="D11">
+        <v>20</v>
+      </c>
+      <c r="E11">
+        <v>80</v>
+      </c>
+      <c r="G11">
+        <v>75</v>
+      </c>
+      <c r="H11">
+        <v>25</v>
+      </c>
+      <c r="I11">
+        <v>8</v>
+      </c>
+      <c r="J11">
+        <v>92</v>
+      </c>
+      <c r="L11">
+        <v>67</v>
+      </c>
+      <c r="M11">
+        <v>33</v>
+      </c>
+      <c r="N11">
+        <v>27</v>
+      </c>
+      <c r="O11">
+        <v>73</v>
+      </c>
+      <c r="Q11">
+        <f t="shared" ref="Q11:Q14" si="6">AVERAGE(C11,D11)</f>
+        <v>17</v>
+      </c>
+      <c r="R11">
+        <f t="shared" ref="R11:R14" si="7">AVERAGE(H11,I11)</f>
+        <v>16.5</v>
+      </c>
+      <c r="S11">
+        <f t="shared" ref="S11:S14" si="8">AVERAGE(M11,N11)</f>
+        <v>30</v>
+      </c>
+      <c r="T11">
+        <f t="shared" ref="T11:T14" si="9">AVERAGE(Q11:S11)</f>
+        <v>21.166666666666668</v>
+      </c>
+      <c r="U11">
+        <f>AVERAGE(Q11:Q16)</f>
+        <v>16.5</v>
+      </c>
+      <c r="V11">
+        <f>_xlfn.STDEV.S(Q11:Q16)</f>
+        <v>0.70710678118654757</v>
+      </c>
+      <c r="W11">
+        <f>AVERAGE(R11:R16)</f>
+        <v>17.25</v>
+      </c>
+      <c r="X11">
+        <f>_xlfn.STDEV.S(R11:R16)</f>
+        <v>3.378855822118882</v>
+      </c>
+      <c r="Y11">
+        <f>AVERAGE(S11:S16)</f>
+        <v>31.25</v>
+      </c>
+      <c r="Z11">
+        <f>_xlfn.STDEV.S(S11:S16)</f>
+        <v>3.1754264805429417</v>
+      </c>
+      <c r="AA11">
+        <f>AVERAGE(T11:T16)</f>
+        <v>21.666666666666668</v>
+      </c>
+      <c r="AB11">
+        <f>_xlfn.STDEV.S(T11:T16)</f>
+        <v>2.2730302828309759</v>
+      </c>
+      <c r="AC11">
+        <f t="shared" ref="AC11:AC14" si="10">MIN(Q11:S11)</f>
+        <v>16.5</v>
+      </c>
+      <c r="AD11">
+        <f t="shared" ref="AD11:AD14" si="11">(T11-AC11)</f>
+        <v>4.6666666666666679</v>
+      </c>
+      <c r="AE11">
+        <f>AVERAGE(AD11:AD16)</f>
+        <v>5.7916666666666679</v>
+      </c>
+      <c r="AF11">
+        <f>_xlfn.STDEV.S(AD11:AD16)</f>
+        <v>1.6007810593582092</v>
+      </c>
+    </row>
+    <row r="12" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B12">
+        <v>95</v>
+      </c>
+      <c r="C12">
+        <v>5</v>
+      </c>
+      <c r="D12">
+        <v>28</v>
+      </c>
+      <c r="E12">
+        <v>72</v>
+      </c>
+      <c r="G12">
+        <v>67</v>
+      </c>
+      <c r="H12">
+        <v>33</v>
+      </c>
+      <c r="I12">
         <v>11</v>
       </c>
-      <c r="R2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S2" t="s">
+      <c r="J12">
+        <v>89</v>
+      </c>
+      <c r="L12">
+        <v>65</v>
+      </c>
+      <c r="M12">
+        <v>35</v>
+      </c>
+      <c r="N12">
+        <v>36</v>
+      </c>
+      <c r="O12">
+        <v>64</v>
+      </c>
+      <c r="Q12">
+        <f t="shared" si="6"/>
+        <v>16.5</v>
+      </c>
+      <c r="R12">
+        <f t="shared" si="7"/>
+        <v>22</v>
+      </c>
+      <c r="S12">
+        <f t="shared" si="8"/>
+        <v>35.5</v>
+      </c>
+      <c r="T12">
+        <f t="shared" si="9"/>
+        <v>24.666666666666668</v>
+      </c>
+      <c r="AC12">
+        <f t="shared" si="10"/>
+        <v>16.5</v>
+      </c>
+      <c r="AD12">
+        <f t="shared" si="11"/>
+        <v>8.1666666666666679</v>
+      </c>
+    </row>
+    <row r="13" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B13">
+        <v>87</v>
+      </c>
+      <c r="C13">
         <v>13</v>
       </c>
-      <c r="T2" t="s">
-        <v>15</v>
-      </c>
-      <c r="U2" t="s">
-        <v>59</v>
-      </c>
-      <c r="V2" t="s">
-        <v>51</v>
-      </c>
-      <c r="W2" t="s">
-        <v>60</v>
-      </c>
-      <c r="X2" t="s">
-        <v>52</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>61</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>1</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AC2" t="s">
+      <c r="D13">
+        <v>18</v>
+      </c>
+      <c r="E13">
+        <v>82</v>
+      </c>
+      <c r="G13">
+        <v>76</v>
+      </c>
+      <c r="H13">
+        <v>24</v>
+      </c>
+      <c r="I13">
+        <v>4</v>
+      </c>
+      <c r="J13">
+        <v>96</v>
+      </c>
+      <c r="L13">
+        <v>70</v>
+      </c>
+      <c r="M13">
+        <v>30</v>
+      </c>
+      <c r="N13">
+        <v>26</v>
+      </c>
+      <c r="O13">
+        <v>74</v>
+      </c>
+      <c r="Q13">
+        <f t="shared" si="6"/>
+        <v>15.5</v>
+      </c>
+      <c r="R13">
+        <f t="shared" si="7"/>
+        <v>14</v>
+      </c>
+      <c r="S13">
+        <f t="shared" si="8"/>
+        <v>28</v>
+      </c>
+      <c r="T13">
+        <f t="shared" si="9"/>
+        <v>19.166666666666668</v>
+      </c>
+      <c r="AC13">
+        <f t="shared" si="10"/>
+        <v>14</v>
+      </c>
+      <c r="AD13">
+        <f t="shared" si="11"/>
+        <v>5.1666666666666679</v>
+      </c>
+    </row>
+    <row r="14" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B14">
+        <v>80</v>
+      </c>
+      <c r="C14">
+        <v>20</v>
+      </c>
+      <c r="D14">
+        <v>14</v>
+      </c>
+      <c r="E14">
+        <v>86</v>
+      </c>
+      <c r="G14">
+        <v>71</v>
+      </c>
+      <c r="H14">
+        <v>29</v>
+      </c>
+      <c r="I14">
+        <v>4</v>
+      </c>
+      <c r="J14">
+        <v>96</v>
+      </c>
+      <c r="L14">
+        <v>62</v>
+      </c>
+      <c r="M14">
+        <v>38</v>
+      </c>
+      <c r="N14">
+        <v>25</v>
+      </c>
+      <c r="O14">
+        <v>75</v>
+      </c>
+      <c r="Q14">
+        <f t="shared" si="6"/>
         <v>17</v>
       </c>
-      <c r="AD2" t="s">
-        <v>14</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>18</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>22</v>
-      </c>
-      <c r="F3" t="s">
-        <v>70</v>
-      </c>
-      <c r="K3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B4">
-        <v>90</v>
-      </c>
-      <c r="C4">
-        <v>10</v>
-      </c>
-      <c r="D4">
-        <v>15</v>
-      </c>
-      <c r="E4">
-        <v>85</v>
-      </c>
-      <c r="G4">
-        <v>61</v>
-      </c>
-      <c r="H4">
-        <v>39</v>
-      </c>
-      <c r="I4">
-        <v>7</v>
-      </c>
-      <c r="J4">
-        <v>93</v>
-      </c>
-      <c r="L4">
-        <v>72</v>
-      </c>
-      <c r="M4">
-        <v>28</v>
-      </c>
-      <c r="N4">
-        <v>20</v>
-      </c>
-      <c r="O4">
-        <v>80</v>
-      </c>
-      <c r="Q4">
-        <f>AVERAGE(C4,D4)</f>
-        <v>12.5</v>
-      </c>
-      <c r="R4">
-        <f>AVERAGE(H4,I4)</f>
-        <v>23</v>
-      </c>
-      <c r="S4">
-        <f>AVERAGE(M4,N4)</f>
-        <v>24</v>
-      </c>
-      <c r="T4">
-        <f>AVERAGE(Q4:S4)</f>
-        <v>19.833333333333332</v>
-      </c>
-      <c r="U4">
-        <f>AVERAGE(Q4:Q10)</f>
-        <v>14.214285714285714</v>
-      </c>
-      <c r="V4">
-        <f>_xlfn.STDEV.S(Q4:Q10)</f>
-        <v>2.0987524639084736</v>
-      </c>
-      <c r="W4">
-        <f>AVERAGE(R4:R10)</f>
-        <v>23</v>
-      </c>
-      <c r="X4">
-        <f>_xlfn.STDEV.S(R4:R10)</f>
-        <v>2.5495097567963922</v>
-      </c>
-      <c r="Y4">
-        <f>AVERAGE(S4:S10)</f>
-        <v>31.428571428571427</v>
-      </c>
-      <c r="Z4">
-        <f>_xlfn.STDEV.S(S4:S10)</f>
-        <v>5.2870011303555522</v>
-      </c>
-      <c r="AA4">
-        <f>AVERAGE(T4:T10)</f>
-        <v>22.88095238095238</v>
-      </c>
-      <c r="AB4">
-        <f>_xlfn.STDEV.S(T4:T10)</f>
-        <v>2.2601914981845255</v>
-      </c>
-      <c r="AC4">
-        <f>MIN(Q4:S4)</f>
-        <v>12.5</v>
-      </c>
-      <c r="AD4">
-        <f>T4-AC4</f>
-        <v>7.3333333333333321</v>
-      </c>
-      <c r="AE4">
-        <f>AVERAGE(AD4:AD10)</f>
-        <v>8.6666666666666661</v>
-      </c>
-      <c r="AF4">
-        <f>_xlfn.STDEV.S(AD4:AD10)</f>
-        <v>2.0971762320196583</v>
-      </c>
-    </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B5">
-        <v>87</v>
-      </c>
-      <c r="C5">
-        <v>13</v>
-      </c>
-      <c r="D5">
-        <v>15</v>
-      </c>
-      <c r="E5">
-        <v>85</v>
-      </c>
-      <c r="G5">
-        <v>49</v>
-      </c>
-      <c r="H5">
-        <v>51</v>
-      </c>
-      <c r="I5">
-        <v>2</v>
-      </c>
-      <c r="J5">
-        <v>98</v>
-      </c>
-      <c r="L5">
-        <v>58</v>
-      </c>
-      <c r="M5">
-        <v>42</v>
-      </c>
-      <c r="N5">
-        <v>25</v>
-      </c>
-      <c r="O5">
-        <v>75</v>
-      </c>
-      <c r="Q5">
-        <f t="shared" ref="Q5:Q10" si="0">AVERAGE(C5,D5)</f>
-        <v>14</v>
-      </c>
-      <c r="R5">
-        <f t="shared" ref="R5:R10" si="1">AVERAGE(H5,I5)</f>
-        <v>26.5</v>
-      </c>
-      <c r="S5">
-        <f t="shared" ref="S5:S10" si="2">AVERAGE(M5,N5)</f>
-        <v>33.5</v>
-      </c>
-      <c r="T5">
-        <f t="shared" ref="T5:T10" si="3">AVERAGE(Q5:S5)</f>
-        <v>24.666666666666668</v>
-      </c>
-      <c r="AC5">
-        <f t="shared" ref="AC5:AC10" si="4">MIN(Q5:S5)</f>
-        <v>14</v>
-      </c>
-      <c r="AD5">
-        <f t="shared" ref="AD5:AD10" si="5">T5-AC5</f>
-        <v>10.666666666666668</v>
-      </c>
-    </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6">
-        <v>84</v>
-      </c>
-      <c r="C6">
-        <v>16</v>
-      </c>
-      <c r="D6">
-        <v>19</v>
-      </c>
-      <c r="E6">
-        <v>81</v>
-      </c>
-      <c r="G6">
-        <v>56</v>
-      </c>
-      <c r="H6">
-        <v>44</v>
-      </c>
-      <c r="I6">
-        <v>8</v>
-      </c>
-      <c r="J6">
-        <v>92</v>
-      </c>
-      <c r="L6">
-        <v>69</v>
-      </c>
-      <c r="M6">
-        <v>31</v>
-      </c>
-      <c r="N6">
-        <v>25</v>
-      </c>
-      <c r="O6">
-        <v>75</v>
-      </c>
-      <c r="Q6">
-        <f t="shared" si="0"/>
-        <v>17.5</v>
-      </c>
-      <c r="R6">
-        <f t="shared" si="1"/>
-        <v>26</v>
-      </c>
-      <c r="S6">
-        <f t="shared" si="2"/>
-        <v>28</v>
-      </c>
-      <c r="T6">
-        <f t="shared" si="3"/>
-        <v>23.833333333333332</v>
-      </c>
-      <c r="AC6">
-        <f t="shared" si="4"/>
-        <v>17.5</v>
-      </c>
-      <c r="AD6">
-        <f t="shared" si="5"/>
-        <v>6.3333333333333321</v>
-      </c>
-    </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B7">
-        <v>90</v>
-      </c>
-      <c r="C7">
-        <v>10</v>
-      </c>
-      <c r="D7">
-        <v>12</v>
-      </c>
-      <c r="E7">
-        <v>88</v>
-      </c>
-      <c r="G7">
-        <v>67</v>
-      </c>
-      <c r="H7">
-        <v>33</v>
-      </c>
-      <c r="I7">
-        <v>8</v>
-      </c>
-      <c r="J7">
-        <v>92</v>
-      </c>
-      <c r="L7">
-        <v>58</v>
-      </c>
-      <c r="M7">
-        <v>42</v>
-      </c>
-      <c r="N7">
-        <v>23</v>
-      </c>
-      <c r="O7">
-        <v>77</v>
-      </c>
-      <c r="Q7">
-        <f t="shared" si="0"/>
-        <v>11</v>
-      </c>
-      <c r="R7">
-        <f t="shared" si="1"/>
-        <v>20.5</v>
-      </c>
-      <c r="S7">
-        <f t="shared" si="2"/>
-        <v>32.5</v>
-      </c>
-      <c r="T7">
-        <f t="shared" si="3"/>
-        <v>21.333333333333332</v>
-      </c>
-      <c r="AC7">
-        <f t="shared" si="4"/>
-        <v>11</v>
-      </c>
-      <c r="AD7">
-        <f t="shared" si="5"/>
-        <v>10.333333333333332</v>
-      </c>
-    </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B8">
-        <v>89</v>
-      </c>
-      <c r="C8">
-        <v>11</v>
-      </c>
-      <c r="D8">
-        <v>19</v>
-      </c>
-      <c r="E8">
-        <v>81</v>
-      </c>
-      <c r="G8">
-        <v>62</v>
-      </c>
-      <c r="H8">
-        <v>38</v>
-      </c>
-      <c r="I8">
-        <v>9</v>
-      </c>
-      <c r="J8">
-        <v>91</v>
-      </c>
-      <c r="L8">
-        <v>52</v>
-      </c>
-      <c r="M8">
-        <v>48</v>
-      </c>
-      <c r="N8">
-        <v>34</v>
-      </c>
-      <c r="O8">
-        <v>66</v>
-      </c>
-      <c r="Q8">
-        <f t="shared" si="0"/>
-        <v>15</v>
-      </c>
-      <c r="R8">
-        <f t="shared" si="1"/>
-        <v>23.5</v>
-      </c>
-      <c r="S8">
-        <f t="shared" si="2"/>
-        <v>41</v>
-      </c>
-      <c r="T8">
-        <f t="shared" si="3"/>
-        <v>26.5</v>
-      </c>
-      <c r="AC8">
-        <f t="shared" si="4"/>
-        <v>15</v>
-      </c>
-      <c r="AD8">
-        <f t="shared" si="5"/>
-        <v>11.5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B9">
-        <v>88</v>
-      </c>
-      <c r="C9">
-        <v>12</v>
-      </c>
-      <c r="D9">
-        <v>16</v>
-      </c>
-      <c r="E9">
-        <v>84</v>
-      </c>
-      <c r="G9">
-        <v>65</v>
-      </c>
-      <c r="H9">
-        <v>35</v>
-      </c>
-      <c r="I9">
-        <v>8</v>
-      </c>
-      <c r="J9">
-        <v>92</v>
-      </c>
-      <c r="L9">
-        <v>65</v>
-      </c>
-      <c r="M9">
-        <v>35</v>
-      </c>
-      <c r="N9">
-        <v>24</v>
-      </c>
-      <c r="O9">
-        <v>76</v>
-      </c>
-      <c r="Q9">
-        <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-      <c r="R9">
-        <f t="shared" si="1"/>
-        <v>21.5</v>
-      </c>
-      <c r="S9">
-        <f t="shared" si="2"/>
-        <v>29.5</v>
-      </c>
-      <c r="T9">
-        <f t="shared" si="3"/>
+      <c r="R14">
+        <f t="shared" si="7"/>
+        <v>16.5</v>
+      </c>
+      <c r="S14">
+        <f t="shared" si="8"/>
+        <v>31.5</v>
+      </c>
+      <c r="T14">
+        <f t="shared" si="9"/>
         <v>21.666666666666668</v>
       </c>
-      <c r="AC9">
-        <f t="shared" si="4"/>
-        <v>14</v>
-      </c>
-      <c r="AD9">
-        <f t="shared" si="5"/>
-        <v>7.6666666666666679</v>
-      </c>
-    </row>
-    <row r="10" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B10">
-        <v>83</v>
-      </c>
-      <c r="C10">
-        <v>17</v>
-      </c>
-      <c r="D10">
-        <v>14</v>
-      </c>
-      <c r="E10">
-        <v>86</v>
-      </c>
-      <c r="G10">
-        <v>64</v>
-      </c>
-      <c r="H10">
-        <v>36</v>
-      </c>
-      <c r="I10">
-        <v>4</v>
-      </c>
-      <c r="J10">
-        <v>96</v>
-      </c>
-      <c r="L10">
-        <v>64</v>
-      </c>
-      <c r="M10">
-        <v>36</v>
-      </c>
-      <c r="N10">
-        <v>27</v>
-      </c>
-      <c r="O10">
-        <v>73</v>
-      </c>
-      <c r="Q10">
-        <f t="shared" si="0"/>
-        <v>15.5</v>
-      </c>
-      <c r="R10">
-        <f t="shared" si="1"/>
-        <v>20</v>
-      </c>
-      <c r="S10">
-        <f t="shared" si="2"/>
-        <v>31.5</v>
-      </c>
-      <c r="T10">
-        <f t="shared" si="3"/>
-        <v>22.333333333333332</v>
-      </c>
-      <c r="AC10">
-        <f t="shared" si="4"/>
-        <v>15.5</v>
-      </c>
-      <c r="AD10">
-        <f t="shared" si="5"/>
-        <v>6.8333333333333321</v>
+      <c r="AC14">
+        <f t="shared" si="10"/>
+        <v>16.5</v>
+      </c>
+      <c r="AD14">
+        <f t="shared" si="11"/>
+        <v>5.1666666666666679</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Trying to see how exp are going
</commit_message>
<xml_diff>
--- a/DataAnalysis/CI/0.05/Results.xlsx
+++ b/DataAnalysis/CI/0.05/Results.xlsx
@@ -8,29 +8,30 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utente\Desktop\CultureAwarenessTest\DataAnalysis\CI\0.05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFD836C5-5436-4C50-9C59-2E78A5A61823}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0BA1E91-2D0C-4A17-9D0E-FC10BF2B56CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
-    <sheet name="MIT_DIFF_ONLYMIN_STDAUG" sheetId="19" r:id="rId2"/>
-    <sheet name="PARBS_STDAUG" sheetId="20" r:id="rId3"/>
-    <sheet name="MIT_DIFF_ONLYMIN_NOAUG" sheetId="18" r:id="rId4"/>
-    <sheet name="MIT_PARBS_DIFF_ONLYMIN_STDAUG" sheetId="17" r:id="rId5"/>
-    <sheet name="MIT_PARBS_STDAUG" sheetId="14" r:id="rId6"/>
-    <sheet name="MIT_DIFF_STDAUG" sheetId="16" r:id="rId7"/>
-    <sheet name="MIT_DIFF_NOAUG" sheetId="15" r:id="rId8"/>
-    <sheet name="MIT_STDAUG" sheetId="12" r:id="rId9"/>
-    <sheet name="MIT_NOAUG" sheetId="11" r:id="rId10"/>
-    <sheet name="MIT_PARBS_NOAUG" sheetId="13" r:id="rId11"/>
-    <sheet name="STD_IMB_AUG" sheetId="10" r:id="rId12"/>
-    <sheet name="STD_IMB_NOAUG" sheetId="9" r:id="rId13"/>
-    <sheet name="DIFF" sheetId="8" r:id="rId14"/>
-    <sheet name="STD_BAL_ADV_NOCLSDIV" sheetId="7" r:id="rId15"/>
-    <sheet name="STD_BAL_ADV_CLSDIV" sheetId="6" r:id="rId16"/>
-    <sheet name="STD_BAL_STDAUG" sheetId="5" r:id="rId17"/>
-    <sheet name="STD_BAL_NOAUG" sheetId="2" r:id="rId18"/>
+    <sheet name="DIFF_ONLYMIN" sheetId="21" r:id="rId2"/>
+    <sheet name="MIT_DIFF_ONLYMIN_STDAUG" sheetId="19" r:id="rId3"/>
+    <sheet name="PARBS_STDAUG" sheetId="20" r:id="rId4"/>
+    <sheet name="MIT_DIFF_ONLYMIN_NOAUG" sheetId="18" r:id="rId5"/>
+    <sheet name="MIT_PARBS_DIFF_ONLYMIN_STDAUG" sheetId="17" r:id="rId6"/>
+    <sheet name="MIT_PARBS_STDAUG" sheetId="14" r:id="rId7"/>
+    <sheet name="MIT_DIFF_STDAUG" sheetId="16" r:id="rId8"/>
+    <sheet name="MIT_DIFF_NOAUG" sheetId="15" r:id="rId9"/>
+    <sheet name="MIT_STDAUG" sheetId="12" r:id="rId10"/>
+    <sheet name="MIT_NOAUG" sheetId="11" r:id="rId11"/>
+    <sheet name="MIT_PARBS_NOAUG" sheetId="13" r:id="rId12"/>
+    <sheet name="STD_IMB_AUG" sheetId="10" r:id="rId13"/>
+    <sheet name="STD_IMB_NOAUG" sheetId="9" r:id="rId14"/>
+    <sheet name="DIFF" sheetId="8" r:id="rId15"/>
+    <sheet name="STD_BAL_ADV_NOCLSDIV" sheetId="7" r:id="rId16"/>
+    <sheet name="STD_BAL_ADV_CLSDIV" sheetId="6" r:id="rId17"/>
+    <sheet name="STD_BAL_STDAUG" sheetId="5" r:id="rId18"/>
+    <sheet name="STD_BAL_NOAUG" sheetId="2" r:id="rId19"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -53,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="85">
   <si>
     <t>Dati originali</t>
   </si>
@@ -305,6 +306,9 @@
   </si>
   <si>
     <t>try</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIFF </t>
   </si>
 </sst>
 </file>
@@ -640,13 +644,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P34"/>
+  <dimension ref="A1:AA36"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -681,12 +685,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
         <v>4</v>
       </c>
@@ -721,7 +725,7 @@
         <v>0.69388866648871195</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
         <v>2</v>
       </c>
@@ -759,17 +763,17 @@
         <v>1.7506612507320798</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="D6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="F7" t="s">
         <v>74</v>
       </c>
@@ -804,12 +808,12 @@
         <v>1.7677669529663689</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="D8" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="F9" t="s">
         <v>74</v>
       </c>
@@ -844,7 +848,7 @@
         <v>3.1819805153394638</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="C10" t="s">
         <v>54</v>
       </c>
@@ -879,7 +883,7 @@
         <v>0.87589712135373932</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
       <c r="C11" t="s">
         <v>82</v>
       </c>
@@ -913,514 +917,584 @@
       <c r="P11">
         <v>1.3402597868683128</v>
       </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="B12" t="s">
+      <c r="R11">
+        <v>16</v>
+      </c>
+      <c r="S11">
+        <v>1.1547005383792515</v>
+      </c>
+      <c r="T11">
+        <v>19.5</v>
+      </c>
+      <c r="U11">
+        <v>2.0816659994661326</v>
+      </c>
+      <c r="V11">
+        <v>30.875</v>
+      </c>
+      <c r="W11">
+        <v>2.5289984842489197</v>
+      </c>
+      <c r="X11">
+        <v>22.125000000000004</v>
+      </c>
+      <c r="Y11">
+        <v>0.41666666666666685</v>
+      </c>
+      <c r="Z11">
+        <v>6.1250000000000009</v>
+      </c>
+      <c r="AA11">
+        <v>0.97539165922663384</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="C12" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="D13" t="s">
+        <v>73</v>
+      </c>
+      <c r="G13">
+        <v>16</v>
+      </c>
+      <c r="H13">
+        <v>1.1547005383792515</v>
+      </c>
+      <c r="I13">
+        <v>19.5</v>
+      </c>
+      <c r="J13">
+        <v>2.0816659994661326</v>
+      </c>
+      <c r="K13">
+        <v>30.875</v>
+      </c>
+      <c r="L13">
+        <v>2.5289984842489197</v>
+      </c>
+      <c r="M13">
+        <v>22.125000000000004</v>
+      </c>
+      <c r="N13">
+        <v>0.41666666666666685</v>
+      </c>
+      <c r="O13">
+        <v>6.1250000000000009</v>
+      </c>
+      <c r="P13">
+        <v>0.97539165922663384</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="B14" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="C13" t="s">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="C15" t="s">
         <v>4</v>
       </c>
-      <c r="G13">
+      <c r="G15">
         <v>17.149999999999999</v>
       </c>
-      <c r="H13">
+      <c r="H15">
         <v>1.8715709384839754</v>
       </c>
-      <c r="I13">
+      <c r="I15">
         <v>21</v>
       </c>
-      <c r="J13">
+      <c r="J15">
         <v>2.4832774042918899</v>
       </c>
-      <c r="K13">
+      <c r="K15">
         <v>31.5</v>
       </c>
-      <c r="L13">
+      <c r="L15">
         <v>3.3499585403736298</v>
       </c>
-      <c r="M13">
+      <c r="M15">
         <v>23.216666666666669</v>
       </c>
-      <c r="N13">
+      <c r="N15">
         <v>1.8510090674821758</v>
       </c>
-      <c r="O13">
+      <c r="O15">
         <v>6.2666666666666657</v>
       </c>
-      <c r="P13">
+      <c r="P15">
         <v>1.354462218459632</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="C15" t="s">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="C17" t="s">
         <v>2</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F17" t="s">
         <v>20</v>
       </c>
-      <c r="G15">
+      <c r="G17">
         <v>17</v>
       </c>
-      <c r="H15">
+      <c r="H17">
         <v>2.8771127502720115</v>
       </c>
-      <c r="I15">
+      <c r="I17">
         <v>19.95</v>
       </c>
-      <c r="J15">
+      <c r="J17">
         <v>1.6741498671796915</v>
       </c>
-      <c r="K15">
+      <c r="K17">
         <v>29.75</v>
       </c>
-      <c r="L15">
+      <c r="L17">
         <v>2.226731535981231</v>
       </c>
-      <c r="M15">
+      <c r="M17">
         <v>22.233333333333327</v>
       </c>
-      <c r="N15">
+      <c r="N17">
         <v>1.3314801936840213</v>
       </c>
-      <c r="O15">
+      <c r="O17">
         <v>5.2833333333333341</v>
       </c>
-      <c r="P15">
+      <c r="P17">
         <v>1.777864581214158</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B17" t="s">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="B19" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="C18" t="s">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="C20" t="s">
         <v>4</v>
       </c>
-      <c r="G18">
+      <c r="G20">
         <v>14.214285714285714</v>
       </c>
-      <c r="H18">
+      <c r="H20">
         <v>2.0987524639084736</v>
       </c>
-      <c r="I18">
+      <c r="I20">
         <v>23</v>
       </c>
-      <c r="J18">
+      <c r="J20">
         <v>2.5495097567963922</v>
       </c>
-      <c r="K18">
+      <c r="K20">
         <v>31.428571428571427</v>
       </c>
-      <c r="L18">
+      <c r="L20">
         <v>5.2870011303555522</v>
       </c>
-      <c r="M18">
+      <c r="M20">
         <v>22.88095238095238</v>
       </c>
-      <c r="N18">
+      <c r="N20">
         <v>2.2601914981845255</v>
       </c>
-      <c r="O18">
+      <c r="O20">
         <v>8.6666666666666661</v>
       </c>
-      <c r="P18">
+      <c r="P20">
         <v>2.0971762320196583</v>
       </c>
     </row>
-    <row r="19" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="C19" t="s">
-        <v>71</v>
-      </c>
-      <c r="F19" t="s">
-        <v>20</v>
-      </c>
-      <c r="G19">
-        <v>14.916666666666666</v>
-      </c>
-      <c r="H19">
-        <v>2.1775368347439388</v>
-      </c>
-      <c r="I19">
-        <v>20.416666666666668</v>
-      </c>
-      <c r="J19">
-        <v>2.4983327774071045</v>
-      </c>
-      <c r="K19">
-        <v>26.416666666666668</v>
-      </c>
-      <c r="L19">
-        <v>1.4288690166235207</v>
-      </c>
-      <c r="M19">
-        <v>20.583333333333332</v>
-      </c>
-      <c r="N19">
-        <v>1.0368220676663862</v>
-      </c>
-      <c r="O19">
-        <v>5.666666666666667</v>
-      </c>
-      <c r="P19">
-        <v>1.7224014243685055</v>
-      </c>
-    </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="C20" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="D21" t="s">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="C21" t="s">
         <v>71</v>
       </c>
       <c r="F21" t="s">
         <v>20</v>
       </c>
       <c r="G21">
+        <v>14.916666666666666</v>
+      </c>
+      <c r="H21">
+        <v>2.1775368347439388</v>
+      </c>
+      <c r="I21">
+        <v>20.416666666666668</v>
+      </c>
+      <c r="J21">
+        <v>2.4983327774071045</v>
+      </c>
+      <c r="K21">
+        <v>26.416666666666668</v>
+      </c>
+      <c r="L21">
+        <v>1.4288690166235207</v>
+      </c>
+      <c r="M21">
+        <v>20.583333333333332</v>
+      </c>
+      <c r="N21">
+        <v>1.0368220676663862</v>
+      </c>
+      <c r="O21">
+        <v>5.666666666666667</v>
+      </c>
+      <c r="P21">
+        <v>1.7224014243685055</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="C22" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="D23" t="s">
+        <v>71</v>
+      </c>
+      <c r="F23" t="s">
+        <v>20</v>
+      </c>
+      <c r="G23">
         <v>18.7</v>
       </c>
-      <c r="H21">
+      <c r="H23">
         <v>2.7748873851023195</v>
       </c>
-      <c r="I21">
+      <c r="I23">
         <v>18.5</v>
       </c>
-      <c r="J21">
+      <c r="J23">
         <v>1.541103500742244</v>
       </c>
-      <c r="K21">
+      <c r="K23">
         <v>27.5</v>
       </c>
-      <c r="L21">
+      <c r="L23">
         <v>1.2247448713915889</v>
       </c>
-      <c r="M21">
+      <c r="M23">
         <v>21.566666666666666</v>
       </c>
-      <c r="N21">
+      <c r="N23">
         <v>1.4841757907262121</v>
       </c>
-      <c r="O21">
+      <c r="O23">
         <v>3.9666666666666663</v>
       </c>
-      <c r="P21">
+      <c r="P23">
         <v>0.74907350180814036</v>
       </c>
     </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="F22" t="s">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="F24" t="s">
         <v>81</v>
       </c>
-      <c r="G22">
+      <c r="G24">
         <v>16.5</v>
       </c>
-      <c r="H22">
+      <c r="H24">
         <v>0.70710678118654757</v>
       </c>
-      <c r="I22">
+      <c r="I24">
         <v>17.25</v>
       </c>
-      <c r="J22">
+      <c r="J24">
         <v>3.378855822118882</v>
       </c>
-      <c r="K22">
+      <c r="K24">
         <v>31.25</v>
       </c>
-      <c r="L22">
+      <c r="L24">
         <v>3.1754264805429417</v>
       </c>
-      <c r="M22">
+      <c r="M24">
         <v>21.6666666666667</v>
       </c>
-      <c r="N22">
+      <c r="N24">
         <v>2.2730302828309759</v>
       </c>
-      <c r="O22">
+      <c r="O24">
         <v>5.7916666666666679</v>
       </c>
-      <c r="P22">
+      <c r="P24">
         <v>1.6007810593582092</v>
       </c>
     </row>
-    <row r="23" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="D23" t="s">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="D25" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="24" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="E24" t="s">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="E26" t="s">
         <v>71</v>
       </c>
-      <c r="G24">
+      <c r="G26">
         <v>15.625</v>
       </c>
-      <c r="H24">
+      <c r="H26">
         <v>1.6007810593582121</v>
       </c>
-      <c r="I24">
+      <c r="I26">
         <v>18.625</v>
       </c>
-      <c r="J24">
+      <c r="J26">
         <v>2.75</v>
       </c>
-      <c r="K24">
+      <c r="K26">
         <v>26.625</v>
       </c>
-      <c r="L24">
+      <c r="L26">
         <v>4.6435439052516774</v>
       </c>
-      <c r="M24">
+      <c r="M26">
         <v>20.291666666666668</v>
       </c>
-      <c r="N24">
+      <c r="N26">
         <v>1.8923579255834544</v>
       </c>
-      <c r="O24">
+      <c r="O26">
         <v>4.791666666666667</v>
       </c>
-      <c r="P24">
+      <c r="P26">
         <v>1.7393858004948073</v>
       </c>
     </row>
-    <row r="25" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="F25" t="s">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="F27" t="s">
         <v>81</v>
       </c>
-      <c r="G25">
+      <c r="G27">
         <v>14.875</v>
       </c>
-      <c r="H25">
+      <c r="H27">
         <v>4.0697051490249265</v>
       </c>
-      <c r="I25">
+      <c r="I27">
         <v>16.5</v>
       </c>
-      <c r="J25">
+      <c r="J27">
         <v>2.2730302828309759</v>
       </c>
-      <c r="K25">
+      <c r="K27">
         <v>27</v>
       </c>
-      <c r="L25">
+      <c r="L27">
         <v>3.3416562759605704</v>
       </c>
-      <c r="M25">
+      <c r="M27">
         <v>19.458333333333332</v>
       </c>
-      <c r="N25">
+      <c r="N27">
         <v>2.1273135553939757</v>
       </c>
-      <c r="O25">
+      <c r="O27">
         <v>5.2083333333333304</v>
       </c>
-      <c r="P25">
+      <c r="P27">
         <v>1.674288129546627</v>
       </c>
     </row>
-    <row r="26" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B26" t="s">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="B28" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="27" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="C27" t="s">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="C29" t="s">
         <v>4</v>
       </c>
-      <c r="G27">
+      <c r="G29">
         <v>16.416666666666668</v>
       </c>
-      <c r="H27">
+      <c r="H29">
         <v>2.8881943609574914</v>
       </c>
-      <c r="I27">
+      <c r="I29">
         <v>15.416666666666666</v>
       </c>
-      <c r="J27">
+      <c r="J29">
         <v>1.2812754062521714</v>
       </c>
-      <c r="K27">
+      <c r="K29">
         <v>29.916666666666668</v>
       </c>
-      <c r="L27">
+      <c r="L29">
         <v>2.437553418218084</v>
       </c>
-      <c r="M27">
+      <c r="M29">
         <v>20.583333333333332</v>
       </c>
-      <c r="N27">
+      <c r="N29">
         <v>1.3570801990548194</v>
       </c>
-      <c r="O27">
+      <c r="O29">
         <v>5.916666666666667</v>
       </c>
-      <c r="P27">
+      <c r="P29">
         <v>1.0527741131569135</v>
       </c>
     </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="C28" t="s">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="C30" t="s">
         <v>71</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F30" t="s">
         <v>20</v>
       </c>
-      <c r="G28">
+      <c r="G30">
         <v>16.8</v>
       </c>
-      <c r="H28">
+      <c r="H30">
         <v>0.57008771254956903</v>
       </c>
-      <c r="I28">
+      <c r="I30">
         <v>17.7</v>
       </c>
-      <c r="J28">
+      <c r="J30">
         <v>1.7175564037317668</v>
       </c>
-      <c r="K28">
+      <c r="K30">
         <v>28.9</v>
       </c>
-      <c r="L28">
+      <c r="L30">
         <v>3.8794329482541587</v>
       </c>
-      <c r="M28">
+      <c r="M30">
         <v>21.133333333333333</v>
       </c>
-      <c r="N28">
+      <c r="N30">
         <v>1.5696779570628134</v>
       </c>
-      <c r="O28">
+      <c r="O30">
         <v>4.7333333333333325</v>
       </c>
-      <c r="P28">
+      <c r="P30">
         <v>0.90215790684828923</v>
       </c>
     </row>
-    <row r="30" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="C30" t="s">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="C32" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="31" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="D31" t="s">
+    <row r="33" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="D33" t="s">
         <v>71</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F33" t="s">
         <v>81</v>
       </c>
-      <c r="G31">
+      <c r="G33">
         <v>16</v>
       </c>
-      <c r="H31">
+      <c r="H33">
         <v>0</v>
       </c>
-      <c r="I31">
+      <c r="I33">
         <v>15.75</v>
       </c>
-      <c r="J31">
+      <c r="J33">
         <v>4.5961940777125587</v>
       </c>
-      <c r="K31">
+      <c r="K33">
         <v>30</v>
       </c>
-      <c r="L31">
+      <c r="L33">
         <v>3.5355339059327378</v>
       </c>
-      <c r="M31">
+      <c r="M33">
         <v>20.583333333333332</v>
       </c>
-      <c r="N31">
+      <c r="N33">
         <v>0.35355339059327379</v>
       </c>
-      <c r="O31">
+      <c r="O33">
         <v>6.3333333333333321</v>
       </c>
-      <c r="P31">
+      <c r="P33">
         <v>2.1213203435596459</v>
       </c>
     </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="D32" t="s">
+    <row r="34" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="D34" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="33" spans="5:16" x14ac:dyDescent="0.3">
-      <c r="E33" t="s">
+    <row r="35" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="E35" t="s">
         <v>71</v>
       </c>
-      <c r="G33">
+      <c r="G35">
         <v>16.375</v>
       </c>
-      <c r="H33">
+      <c r="H35">
         <v>3.3008837200563934</v>
       </c>
-      <c r="I33">
+      <c r="I35">
         <v>20</v>
       </c>
-      <c r="J33">
+      <c r="J35">
         <v>3.3166247903553998</v>
       </c>
-      <c r="K33">
+      <c r="K35">
         <v>26.875</v>
       </c>
-      <c r="L33">
+      <c r="L35">
         <v>1.796988221070652</v>
       </c>
-      <c r="M33">
+      <c r="M35">
         <v>21.083333333333332</v>
       </c>
-      <c r="N33">
+      <c r="N35">
         <v>1.5898986690282424</v>
       </c>
-      <c r="O33">
+      <c r="O35">
         <v>4.708333333333333</v>
       </c>
-      <c r="P33">
+      <c r="P35">
         <v>2.9071272570854019</v>
       </c>
     </row>
-    <row r="34" spans="5:16" x14ac:dyDescent="0.3">
-      <c r="F34" t="s">
+    <row r="36" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="F36" t="s">
         <v>81</v>
       </c>
-      <c r="G34">
+      <c r="G36">
         <v>14.333333333333334</v>
       </c>
-      <c r="H34">
+      <c r="H36">
         <v>3.2145502536643153</v>
       </c>
-      <c r="I34">
+      <c r="I36">
         <v>17.166666666666668</v>
       </c>
-      <c r="J34">
+      <c r="J36">
         <v>1.2583057392117916</v>
       </c>
-      <c r="K34">
+      <c r="K36">
         <v>26.6666666666667</v>
       </c>
-      <c r="L34">
+      <c r="L36">
         <v>4.1633319989322564</v>
       </c>
-      <c r="M34">
+      <c r="M36">
         <v>19.3888888888889</v>
       </c>
-      <c r="N34">
+      <c r="N36">
         <v>2.4962935487400935</v>
       </c>
-      <c r="O34">
+      <c r="O36">
         <v>5.0555555555555562</v>
       </c>
-      <c r="P34">
+      <c r="P36">
         <v>1.3977495139343468</v>
       </c>
     </row>
@@ -1431,6 +1505,785 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25FCA91D-5E11-4BE7-9F8B-616A902FA88F}">
+  <dimension ref="A2:AF14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="2" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>11</v>
+      </c>
+      <c r="R2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S2" t="s">
+        <v>13</v>
+      </c>
+      <c r="T2" t="s">
+        <v>15</v>
+      </c>
+      <c r="U2" t="s">
+        <v>59</v>
+      </c>
+      <c r="V2" t="s">
+        <v>51</v>
+      </c>
+      <c r="W2" t="s">
+        <v>60</v>
+      </c>
+      <c r="X2" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>14</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>18</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s">
+        <v>70</v>
+      </c>
+      <c r="K3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B4">
+        <v>85</v>
+      </c>
+      <c r="C4">
+        <v>15</v>
+      </c>
+      <c r="D4">
+        <v>10</v>
+      </c>
+      <c r="E4">
+        <v>90</v>
+      </c>
+      <c r="G4">
+        <v>72</v>
+      </c>
+      <c r="H4">
+        <v>28</v>
+      </c>
+      <c r="I4">
+        <v>12</v>
+      </c>
+      <c r="J4">
+        <v>88</v>
+      </c>
+      <c r="L4">
+        <v>68</v>
+      </c>
+      <c r="M4">
+        <v>32</v>
+      </c>
+      <c r="N4">
+        <v>25</v>
+      </c>
+      <c r="O4">
+        <v>75</v>
+      </c>
+      <c r="Q4">
+        <f>AVERAGE(C4,D4)</f>
+        <v>12.5</v>
+      </c>
+      <c r="R4">
+        <f>AVERAGE(H4,I4)</f>
+        <v>20</v>
+      </c>
+      <c r="S4">
+        <f>AVERAGE(M4,N4)</f>
+        <v>28.5</v>
+      </c>
+      <c r="T4">
+        <f>AVERAGE(Q4:S4)</f>
+        <v>20.333333333333332</v>
+      </c>
+      <c r="U4">
+        <f>AVERAGE(Q4:Q9)</f>
+        <v>14.916666666666666</v>
+      </c>
+      <c r="V4">
+        <f>_xlfn.STDEV.S(Q4:Q9)</f>
+        <v>2.1775368347439388</v>
+      </c>
+      <c r="W4">
+        <f>AVERAGE(R4:R9)</f>
+        <v>20.416666666666668</v>
+      </c>
+      <c r="X4">
+        <f>_xlfn.STDEV.S(R4:R9)</f>
+        <v>2.4983327774071045</v>
+      </c>
+      <c r="Y4">
+        <f>AVERAGE(S4:S9)</f>
+        <v>26.416666666666668</v>
+      </c>
+      <c r="Z4">
+        <f>_xlfn.STDEV.S(S4:S9)</f>
+        <v>1.4288690166235207</v>
+      </c>
+      <c r="AA4">
+        <f>AVERAGE(T4:T9)</f>
+        <v>20.583333333333332</v>
+      </c>
+      <c r="AB4">
+        <f>_xlfn.STDEV.S(T4:T9)</f>
+        <v>1.0368220676663862</v>
+      </c>
+      <c r="AC4">
+        <f>MIN(Q4:S4)</f>
+        <v>12.5</v>
+      </c>
+      <c r="AD4">
+        <f>(T4-AC4)</f>
+        <v>7.8333333333333321</v>
+      </c>
+      <c r="AE4">
+        <f>AVERAGE(AD4:AD9)</f>
+        <v>5.666666666666667</v>
+      </c>
+      <c r="AF4">
+        <f>_xlfn.STDEV.S(AD4:AD9)</f>
+        <v>1.7224014243685055</v>
+      </c>
+    </row>
+    <row r="5" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B5">
+        <v>88</v>
+      </c>
+      <c r="C5">
+        <v>12</v>
+      </c>
+      <c r="D5">
+        <v>20</v>
+      </c>
+      <c r="E5">
+        <v>80</v>
+      </c>
+      <c r="G5">
+        <v>71</v>
+      </c>
+      <c r="H5">
+        <v>29</v>
+      </c>
+      <c r="I5">
+        <v>5</v>
+      </c>
+      <c r="J5">
+        <v>95</v>
+      </c>
+      <c r="L5">
+        <v>67</v>
+      </c>
+      <c r="M5">
+        <v>33</v>
+      </c>
+      <c r="N5">
+        <v>18</v>
+      </c>
+      <c r="O5">
+        <v>82</v>
+      </c>
+      <c r="Q5">
+        <f t="shared" ref="Q5:Q9" si="0">AVERAGE(C5,D5)</f>
+        <v>16</v>
+      </c>
+      <c r="R5">
+        <f t="shared" ref="R5:R9" si="1">AVERAGE(H5,I5)</f>
+        <v>17</v>
+      </c>
+      <c r="S5">
+        <f t="shared" ref="S5:S9" si="2">AVERAGE(M5,N5)</f>
+        <v>25.5</v>
+      </c>
+      <c r="T5">
+        <f t="shared" ref="T5:T9" si="3">AVERAGE(Q5:S5)</f>
+        <v>19.5</v>
+      </c>
+      <c r="AC5">
+        <f t="shared" ref="AC5:AC9" si="4">MIN(Q5:S5)</f>
+        <v>16</v>
+      </c>
+      <c r="AD5">
+        <f t="shared" ref="AD5:AD9" si="5">(T5-AC5)</f>
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B6">
+        <v>92</v>
+      </c>
+      <c r="C6">
+        <v>8</v>
+      </c>
+      <c r="D6">
+        <v>21</v>
+      </c>
+      <c r="E6">
+        <v>79</v>
+      </c>
+      <c r="G6">
+        <v>78</v>
+      </c>
+      <c r="H6">
+        <v>22</v>
+      </c>
+      <c r="I6">
+        <v>15</v>
+      </c>
+      <c r="J6">
+        <v>85</v>
+      </c>
+      <c r="L6">
+        <v>62</v>
+      </c>
+      <c r="M6">
+        <v>38</v>
+      </c>
+      <c r="N6">
+        <v>18</v>
+      </c>
+      <c r="O6">
+        <v>82</v>
+      </c>
+      <c r="Q6">
+        <f t="shared" si="0"/>
+        <v>14.5</v>
+      </c>
+      <c r="R6">
+        <f t="shared" si="1"/>
+        <v>18.5</v>
+      </c>
+      <c r="S6">
+        <f t="shared" si="2"/>
+        <v>28</v>
+      </c>
+      <c r="T6">
+        <f t="shared" si="3"/>
+        <v>20.333333333333332</v>
+      </c>
+      <c r="AC6">
+        <f t="shared" si="4"/>
+        <v>14.5</v>
+      </c>
+      <c r="AD6">
+        <f t="shared" si="5"/>
+        <v>5.8333333333333321</v>
+      </c>
+    </row>
+    <row r="7" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B7">
+        <v>81</v>
+      </c>
+      <c r="C7">
+        <v>19</v>
+      </c>
+      <c r="D7">
+        <v>13</v>
+      </c>
+      <c r="E7">
+        <v>87</v>
+      </c>
+      <c r="G7">
+        <v>65</v>
+      </c>
+      <c r="H7">
+        <v>35</v>
+      </c>
+      <c r="I7">
+        <v>7</v>
+      </c>
+      <c r="J7">
+        <v>93</v>
+      </c>
+      <c r="L7">
+        <v>67</v>
+      </c>
+      <c r="M7">
+        <v>33</v>
+      </c>
+      <c r="N7">
+        <v>18</v>
+      </c>
+      <c r="O7">
+        <v>82</v>
+      </c>
+      <c r="Q7">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="R7">
+        <f t="shared" si="1"/>
+        <v>21</v>
+      </c>
+      <c r="S7">
+        <f t="shared" si="2"/>
+        <v>25.5</v>
+      </c>
+      <c r="T7">
+        <f t="shared" si="3"/>
+        <v>20.833333333333332</v>
+      </c>
+      <c r="AC7">
+        <f t="shared" si="4"/>
+        <v>16</v>
+      </c>
+      <c r="AD7">
+        <f t="shared" si="5"/>
+        <v>4.8333333333333321</v>
+      </c>
+    </row>
+    <row r="8" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B8">
+        <v>80</v>
+      </c>
+      <c r="C8">
+        <v>20</v>
+      </c>
+      <c r="D8">
+        <v>16</v>
+      </c>
+      <c r="E8">
+        <v>84</v>
+      </c>
+      <c r="G8">
+        <v>60</v>
+      </c>
+      <c r="H8">
+        <v>40</v>
+      </c>
+      <c r="I8">
+        <v>8</v>
+      </c>
+      <c r="J8">
+        <v>92</v>
+      </c>
+      <c r="L8">
+        <v>66</v>
+      </c>
+      <c r="M8">
+        <v>34</v>
+      </c>
+      <c r="N8">
+        <v>17</v>
+      </c>
+      <c r="O8">
+        <v>83</v>
+      </c>
+      <c r="Q8">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="R8">
+        <f t="shared" si="1"/>
+        <v>24</v>
+      </c>
+      <c r="S8">
+        <f t="shared" si="2"/>
+        <v>25.5</v>
+      </c>
+      <c r="T8">
+        <f t="shared" si="3"/>
+        <v>22.5</v>
+      </c>
+      <c r="AC8">
+        <f t="shared" si="4"/>
+        <v>18</v>
+      </c>
+      <c r="AD8">
+        <f t="shared" si="5"/>
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B9">
+        <v>91</v>
+      </c>
+      <c r="C9">
+        <v>9</v>
+      </c>
+      <c r="D9">
+        <v>16</v>
+      </c>
+      <c r="E9">
+        <v>84</v>
+      </c>
+      <c r="G9">
+        <v>66</v>
+      </c>
+      <c r="H9">
+        <v>34</v>
+      </c>
+      <c r="I9">
+        <v>10</v>
+      </c>
+      <c r="J9">
+        <v>90</v>
+      </c>
+      <c r="L9">
+        <v>68</v>
+      </c>
+      <c r="M9">
+        <v>32</v>
+      </c>
+      <c r="N9">
+        <v>19</v>
+      </c>
+      <c r="O9">
+        <v>81</v>
+      </c>
+      <c r="Q9">
+        <f t="shared" si="0"/>
+        <v>12.5</v>
+      </c>
+      <c r="R9">
+        <f t="shared" si="1"/>
+        <v>22</v>
+      </c>
+      <c r="S9">
+        <f t="shared" si="2"/>
+        <v>25.5</v>
+      </c>
+      <c r="T9">
+        <f t="shared" si="3"/>
+        <v>20</v>
+      </c>
+      <c r="AC9">
+        <f t="shared" si="4"/>
+        <v>12.5</v>
+      </c>
+      <c r="AD9">
+        <f t="shared" si="5"/>
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="11" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B11">
+        <v>86</v>
+      </c>
+      <c r="C11">
+        <v>14</v>
+      </c>
+      <c r="D11">
+        <v>20</v>
+      </c>
+      <c r="E11">
+        <v>80</v>
+      </c>
+      <c r="G11">
+        <v>75</v>
+      </c>
+      <c r="H11">
+        <v>25</v>
+      </c>
+      <c r="I11">
+        <v>8</v>
+      </c>
+      <c r="J11">
+        <v>92</v>
+      </c>
+      <c r="L11">
+        <v>67</v>
+      </c>
+      <c r="M11">
+        <v>33</v>
+      </c>
+      <c r="N11">
+        <v>27</v>
+      </c>
+      <c r="O11">
+        <v>73</v>
+      </c>
+      <c r="Q11">
+        <f t="shared" ref="Q11:Q14" si="6">AVERAGE(C11,D11)</f>
+        <v>17</v>
+      </c>
+      <c r="R11">
+        <f t="shared" ref="R11:R14" si="7">AVERAGE(H11,I11)</f>
+        <v>16.5</v>
+      </c>
+      <c r="S11">
+        <f t="shared" ref="S11:S14" si="8">AVERAGE(M11,N11)</f>
+        <v>30</v>
+      </c>
+      <c r="T11">
+        <f t="shared" ref="T11:T14" si="9">AVERAGE(Q11:S11)</f>
+        <v>21.166666666666668</v>
+      </c>
+      <c r="U11">
+        <f>AVERAGE(Q11:Q16)</f>
+        <v>16.5</v>
+      </c>
+      <c r="V11">
+        <f>_xlfn.STDEV.S(Q11:Q16)</f>
+        <v>0.70710678118654757</v>
+      </c>
+      <c r="W11">
+        <f>AVERAGE(R11:R16)</f>
+        <v>17.25</v>
+      </c>
+      <c r="X11">
+        <f>_xlfn.STDEV.S(R11:R16)</f>
+        <v>3.378855822118882</v>
+      </c>
+      <c r="Y11">
+        <f>AVERAGE(S11:S16)</f>
+        <v>31.25</v>
+      </c>
+      <c r="Z11">
+        <f>_xlfn.STDEV.S(S11:S16)</f>
+        <v>3.1754264805429417</v>
+      </c>
+      <c r="AA11">
+        <f>AVERAGE(T11:T16)</f>
+        <v>21.666666666666668</v>
+      </c>
+      <c r="AB11">
+        <f>_xlfn.STDEV.S(T11:T16)</f>
+        <v>2.2730302828309759</v>
+      </c>
+      <c r="AC11">
+        <f t="shared" ref="AC11:AC14" si="10">MIN(Q11:S11)</f>
+        <v>16.5</v>
+      </c>
+      <c r="AD11">
+        <f t="shared" ref="AD11:AD14" si="11">(T11-AC11)</f>
+        <v>4.6666666666666679</v>
+      </c>
+      <c r="AE11">
+        <f>AVERAGE(AD11:AD16)</f>
+        <v>5.7916666666666679</v>
+      </c>
+      <c r="AF11">
+        <f>_xlfn.STDEV.S(AD11:AD16)</f>
+        <v>1.6007810593582092</v>
+      </c>
+    </row>
+    <row r="12" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B12">
+        <v>95</v>
+      </c>
+      <c r="C12">
+        <v>5</v>
+      </c>
+      <c r="D12">
+        <v>28</v>
+      </c>
+      <c r="E12">
+        <v>72</v>
+      </c>
+      <c r="G12">
+        <v>67</v>
+      </c>
+      <c r="H12">
+        <v>33</v>
+      </c>
+      <c r="I12">
+        <v>11</v>
+      </c>
+      <c r="J12">
+        <v>89</v>
+      </c>
+      <c r="L12">
+        <v>65</v>
+      </c>
+      <c r="M12">
+        <v>35</v>
+      </c>
+      <c r="N12">
+        <v>36</v>
+      </c>
+      <c r="O12">
+        <v>64</v>
+      </c>
+      <c r="Q12">
+        <f t="shared" si="6"/>
+        <v>16.5</v>
+      </c>
+      <c r="R12">
+        <f t="shared" si="7"/>
+        <v>22</v>
+      </c>
+      <c r="S12">
+        <f t="shared" si="8"/>
+        <v>35.5</v>
+      </c>
+      <c r="T12">
+        <f t="shared" si="9"/>
+        <v>24.666666666666668</v>
+      </c>
+      <c r="AC12">
+        <f t="shared" si="10"/>
+        <v>16.5</v>
+      </c>
+      <c r="AD12">
+        <f t="shared" si="11"/>
+        <v>8.1666666666666679</v>
+      </c>
+    </row>
+    <row r="13" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B13">
+        <v>87</v>
+      </c>
+      <c r="C13">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>18</v>
+      </c>
+      <c r="E13">
+        <v>82</v>
+      </c>
+      <c r="G13">
+        <v>76</v>
+      </c>
+      <c r="H13">
+        <v>24</v>
+      </c>
+      <c r="I13">
+        <v>4</v>
+      </c>
+      <c r="J13">
+        <v>96</v>
+      </c>
+      <c r="L13">
+        <v>70</v>
+      </c>
+      <c r="M13">
+        <v>30</v>
+      </c>
+      <c r="N13">
+        <v>26</v>
+      </c>
+      <c r="O13">
+        <v>74</v>
+      </c>
+      <c r="Q13">
+        <f t="shared" si="6"/>
+        <v>15.5</v>
+      </c>
+      <c r="R13">
+        <f t="shared" si="7"/>
+        <v>14</v>
+      </c>
+      <c r="S13">
+        <f t="shared" si="8"/>
+        <v>28</v>
+      </c>
+      <c r="T13">
+        <f t="shared" si="9"/>
+        <v>19.166666666666668</v>
+      </c>
+      <c r="AC13">
+        <f t="shared" si="10"/>
+        <v>14</v>
+      </c>
+      <c r="AD13">
+        <f t="shared" si="11"/>
+        <v>5.1666666666666679</v>
+      </c>
+    </row>
+    <row r="14" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="B14">
+        <v>80</v>
+      </c>
+      <c r="C14">
+        <v>20</v>
+      </c>
+      <c r="D14">
+        <v>14</v>
+      </c>
+      <c r="E14">
+        <v>86</v>
+      </c>
+      <c r="G14">
+        <v>71</v>
+      </c>
+      <c r="H14">
+        <v>29</v>
+      </c>
+      <c r="I14">
+        <v>4</v>
+      </c>
+      <c r="J14">
+        <v>96</v>
+      </c>
+      <c r="L14">
+        <v>62</v>
+      </c>
+      <c r="M14">
+        <v>38</v>
+      </c>
+      <c r="N14">
+        <v>25</v>
+      </c>
+      <c r="O14">
+        <v>75</v>
+      </c>
+      <c r="Q14">
+        <f t="shared" si="6"/>
+        <v>17</v>
+      </c>
+      <c r="R14">
+        <f t="shared" si="7"/>
+        <v>16.5</v>
+      </c>
+      <c r="S14">
+        <f t="shared" si="8"/>
+        <v>31.5</v>
+      </c>
+      <c r="T14">
+        <f t="shared" si="9"/>
+        <v>21.666666666666668</v>
+      </c>
+      <c r="AC14">
+        <f t="shared" si="10"/>
+        <v>16.5</v>
+      </c>
+      <c r="AD14">
+        <f t="shared" si="11"/>
+        <v>5.1666666666666679</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8328B926-3ADF-46D7-8F68-CEFFC1D24F6E}">
   <dimension ref="A2:AF10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1981,7 +2834,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEC9CF4A-6F3D-4BA0-B506-17E3C93FB04B}">
   <dimension ref="A2:AF9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2470,7 +3323,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84CA6F53-9387-444E-890F-DCD3D83EC80C}">
   <dimension ref="A1:AO99"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -5309,7 +6162,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C39A647-64D8-47BC-AD52-3FB80D45AD9F}">
   <dimension ref="A1:AG11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -6041,7 +6894,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F319F6D0-ABAC-48C6-A867-062B0035D0C5}">
   <dimension ref="A2:AF15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -6896,7 +7749,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76F82D8A-1A23-4CF3-9872-DA5B576CDAF9}">
   <dimension ref="A1:AN41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -8333,7 +9186,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8214124B-224B-4F9B-B528-181D112DB9C5}">
   <dimension ref="A1:AL41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -9410,7 +10263,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03D9506E-E2C3-4105-A101-2ED902EAE848}">
   <dimension ref="A1:AR109"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -10199,6 +11052,11 @@
         <v>6.3333333333333321</v>
       </c>
     </row>
+    <row r="21" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>81</v>
+      </c>
+    </row>
     <row r="26" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>25</v>
@@ -11946,7 +12804,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D80BAE23-A740-4698-B840-F018E78CD098}">
   <dimension ref="A1:AF5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -12245,6 +13103,354 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74B1D148-F1AF-4FC9-8C19-77A1A130E3CB}">
+  <dimension ref="B2:AF7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="2" spans="2:32" x14ac:dyDescent="0.3">
+      <c r="Q2" t="s">
+        <v>11</v>
+      </c>
+      <c r="R2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S2" t="s">
+        <v>13</v>
+      </c>
+      <c r="T2" t="s">
+        <v>15</v>
+      </c>
+      <c r="U2" t="s">
+        <v>59</v>
+      </c>
+      <c r="V2" t="s">
+        <v>51</v>
+      </c>
+      <c r="W2" t="s">
+        <v>60</v>
+      </c>
+      <c r="X2" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>14</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>18</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="2:32" x14ac:dyDescent="0.3">
+      <c r="B4">
+        <v>86</v>
+      </c>
+      <c r="C4">
+        <v>14</v>
+      </c>
+      <c r="D4">
+        <v>20</v>
+      </c>
+      <c r="E4">
+        <v>80</v>
+      </c>
+      <c r="G4">
+        <v>72</v>
+      </c>
+      <c r="H4">
+        <v>28</v>
+      </c>
+      <c r="I4">
+        <v>10</v>
+      </c>
+      <c r="J4">
+        <v>90</v>
+      </c>
+      <c r="L4">
+        <v>66</v>
+      </c>
+      <c r="M4">
+        <v>34</v>
+      </c>
+      <c r="N4">
+        <v>26</v>
+      </c>
+      <c r="O4">
+        <v>74</v>
+      </c>
+      <c r="Q4">
+        <f>AVERAGE(C4:D4)</f>
+        <v>17</v>
+      </c>
+      <c r="R4">
+        <f>AVERAGE(H4:I4)</f>
+        <v>19</v>
+      </c>
+      <c r="S4">
+        <f>AVERAGE(M4:N4)</f>
+        <v>30</v>
+      </c>
+      <c r="T4">
+        <f>AVERAGE(Q4:S4)</f>
+        <v>22</v>
+      </c>
+      <c r="U4">
+        <f>AVERAGE(Q4:Q7)</f>
+        <v>16</v>
+      </c>
+      <c r="V4">
+        <f>_xlfn.STDEV.S(Q4:Q7)</f>
+        <v>1.1547005383792515</v>
+      </c>
+      <c r="W4">
+        <f>AVERAGE(R4:R7)</f>
+        <v>19.5</v>
+      </c>
+      <c r="X4">
+        <f>_xlfn.STDEV.S(R4:R7)</f>
+        <v>2.0816659994661326</v>
+      </c>
+      <c r="Y4">
+        <f>AVERAGE(S4:S7)</f>
+        <v>30.875</v>
+      </c>
+      <c r="Z4">
+        <f>_xlfn.STDEV.S(S4:S7)</f>
+        <v>2.5289984842489197</v>
+      </c>
+      <c r="AA4">
+        <f>AVERAGE(T4:T7)</f>
+        <v>22.125000000000004</v>
+      </c>
+      <c r="AB4">
+        <f>_xlfn.STDEV.S(T4:T7)</f>
+        <v>0.41666666666666685</v>
+      </c>
+      <c r="AC4">
+        <f>MIN(Q4:S4)</f>
+        <v>17</v>
+      </c>
+      <c r="AD4">
+        <f>T4-AC4</f>
+        <v>5</v>
+      </c>
+      <c r="AE4">
+        <f>AVERAGE(AD4:AD7)</f>
+        <v>6.1250000000000009</v>
+      </c>
+      <c r="AF4">
+        <f>_xlfn.STDEV.S(AD4:AD7)</f>
+        <v>0.97539165922663384</v>
+      </c>
+    </row>
+    <row r="5" spans="2:32" x14ac:dyDescent="0.3">
+      <c r="B5">
+        <v>81</v>
+      </c>
+      <c r="C5">
+        <v>19</v>
+      </c>
+      <c r="D5">
+        <v>11</v>
+      </c>
+      <c r="E5">
+        <v>89</v>
+      </c>
+      <c r="G5">
+        <v>71</v>
+      </c>
+      <c r="H5">
+        <v>29</v>
+      </c>
+      <c r="I5">
+        <v>11</v>
+      </c>
+      <c r="J5">
+        <v>89</v>
+      </c>
+      <c r="L5">
+        <v>55</v>
+      </c>
+      <c r="M5">
+        <v>45</v>
+      </c>
+      <c r="N5">
+        <v>18</v>
+      </c>
+      <c r="O5">
+        <v>82</v>
+      </c>
+      <c r="Q5">
+        <f t="shared" ref="Q5:Q7" si="0">AVERAGE(C5:D5)</f>
+        <v>15</v>
+      </c>
+      <c r="R5">
+        <f t="shared" ref="R5:R7" si="1">AVERAGE(H5:I5)</f>
+        <v>20</v>
+      </c>
+      <c r="S5">
+        <f t="shared" ref="S5:S7" si="2">AVERAGE(M5:N5)</f>
+        <v>31.5</v>
+      </c>
+      <c r="T5">
+        <f t="shared" ref="T5:T7" si="3">AVERAGE(Q5:S5)</f>
+        <v>22.166666666666668</v>
+      </c>
+      <c r="AC5">
+        <f t="shared" ref="AC5:AC7" si="4">MIN(Q5:S5)</f>
+        <v>15</v>
+      </c>
+      <c r="AD5">
+        <f t="shared" ref="AD5:AD7" si="5">T5-AC5</f>
+        <v>7.1666666666666679</v>
+      </c>
+    </row>
+    <row r="6" spans="2:32" x14ac:dyDescent="0.3">
+      <c r="B6">
+        <v>82</v>
+      </c>
+      <c r="C6">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>16</v>
+      </c>
+      <c r="E6">
+        <v>84</v>
+      </c>
+      <c r="G6">
+        <v>69</v>
+      </c>
+      <c r="H6">
+        <v>31</v>
+      </c>
+      <c r="I6">
+        <v>3</v>
+      </c>
+      <c r="J6">
+        <v>97</v>
+      </c>
+      <c r="L6">
+        <v>53</v>
+      </c>
+      <c r="M6">
+        <v>47</v>
+      </c>
+      <c r="N6">
+        <v>21</v>
+      </c>
+      <c r="O6">
+        <v>79</v>
+      </c>
+      <c r="Q6">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="R6">
+        <f t="shared" si="1"/>
+        <v>17</v>
+      </c>
+      <c r="S6">
+        <f t="shared" si="2"/>
+        <v>34</v>
+      </c>
+      <c r="T6">
+        <f t="shared" si="3"/>
+        <v>22.666666666666668</v>
+      </c>
+      <c r="AC6">
+        <f t="shared" si="4"/>
+        <v>17</v>
+      </c>
+      <c r="AD6">
+        <f t="shared" si="5"/>
+        <v>5.6666666666666679</v>
+      </c>
+    </row>
+    <row r="7" spans="2:32" x14ac:dyDescent="0.3">
+      <c r="B7">
+        <v>86</v>
+      </c>
+      <c r="C7">
+        <v>14</v>
+      </c>
+      <c r="D7">
+        <v>16</v>
+      </c>
+      <c r="E7">
+        <v>84</v>
+      </c>
+      <c r="G7">
+        <v>63</v>
+      </c>
+      <c r="H7">
+        <v>37</v>
+      </c>
+      <c r="I7">
+        <v>7</v>
+      </c>
+      <c r="J7">
+        <v>93</v>
+      </c>
+      <c r="L7">
+        <v>65</v>
+      </c>
+      <c r="M7">
+        <v>35</v>
+      </c>
+      <c r="N7">
+        <v>21</v>
+      </c>
+      <c r="O7">
+        <v>79</v>
+      </c>
+      <c r="Q7">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="R7">
+        <f t="shared" si="1"/>
+        <v>22</v>
+      </c>
+      <c r="S7">
+        <f t="shared" si="2"/>
+        <v>28</v>
+      </c>
+      <c r="T7">
+        <f t="shared" si="3"/>
+        <v>21.666666666666668</v>
+      </c>
+      <c r="AC7">
+        <f t="shared" si="4"/>
+        <v>15</v>
+      </c>
+      <c r="AD7">
+        <f t="shared" si="5"/>
+        <v>6.6666666666666679</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D0CE18A-8B26-4E93-B497-B59E55EFEC0E}">
   <dimension ref="A2:AF13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -12902,7 +14108,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1341680-B8DF-484F-AD8E-90C5FE6FD057}">
   <dimension ref="B1:AF3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -13126,7 +14332,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E557A7D-364E-47EE-A0F3-0D888512E587}">
   <dimension ref="A2:AF5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -13292,7 +14498,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1B67D71-588A-4985-8ACA-35F7A9B1AF58}">
   <dimension ref="A2:AF12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -13888,7 +15094,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A366D673-4552-407C-AD95-3B60150A1024}">
   <dimension ref="A2:AF8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -14312,7 +15518,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A4C68C5-0EAB-4233-98F5-D346BC512EB4}">
   <dimension ref="A2:AF31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -15950,7 +17156,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0843B137-6F6F-47C7-80DB-2FF2B4BCD957}">
   <dimension ref="A2:AF5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -16111,783 +17317,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25FCA91D-5E11-4BE7-9F8B-616A902FA88F}">
-  <dimension ref="A2:AF14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>11</v>
-      </c>
-      <c r="R2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S2" t="s">
-        <v>13</v>
-      </c>
-      <c r="T2" t="s">
-        <v>15</v>
-      </c>
-      <c r="U2" t="s">
-        <v>59</v>
-      </c>
-      <c r="V2" t="s">
-        <v>51</v>
-      </c>
-      <c r="W2" t="s">
-        <v>60</v>
-      </c>
-      <c r="X2" t="s">
-        <v>52</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>61</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>1</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>14</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>18</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>22</v>
-      </c>
-      <c r="F3" t="s">
-        <v>70</v>
-      </c>
-      <c r="K3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B4">
-        <v>85</v>
-      </c>
-      <c r="C4">
-        <v>15</v>
-      </c>
-      <c r="D4">
-        <v>10</v>
-      </c>
-      <c r="E4">
-        <v>90</v>
-      </c>
-      <c r="G4">
-        <v>72</v>
-      </c>
-      <c r="H4">
-        <v>28</v>
-      </c>
-      <c r="I4">
-        <v>12</v>
-      </c>
-      <c r="J4">
-        <v>88</v>
-      </c>
-      <c r="L4">
-        <v>68</v>
-      </c>
-      <c r="M4">
-        <v>32</v>
-      </c>
-      <c r="N4">
-        <v>25</v>
-      </c>
-      <c r="O4">
-        <v>75</v>
-      </c>
-      <c r="Q4">
-        <f>AVERAGE(C4,D4)</f>
-        <v>12.5</v>
-      </c>
-      <c r="R4">
-        <f>AVERAGE(H4,I4)</f>
-        <v>20</v>
-      </c>
-      <c r="S4">
-        <f>AVERAGE(M4,N4)</f>
-        <v>28.5</v>
-      </c>
-      <c r="T4">
-        <f>AVERAGE(Q4:S4)</f>
-        <v>20.333333333333332</v>
-      </c>
-      <c r="U4">
-        <f>AVERAGE(Q4:Q9)</f>
-        <v>14.916666666666666</v>
-      </c>
-      <c r="V4">
-        <f>_xlfn.STDEV.S(Q4:Q9)</f>
-        <v>2.1775368347439388</v>
-      </c>
-      <c r="W4">
-        <f>AVERAGE(R4:R9)</f>
-        <v>20.416666666666668</v>
-      </c>
-      <c r="X4">
-        <f>_xlfn.STDEV.S(R4:R9)</f>
-        <v>2.4983327774071045</v>
-      </c>
-      <c r="Y4">
-        <f>AVERAGE(S4:S9)</f>
-        <v>26.416666666666668</v>
-      </c>
-      <c r="Z4">
-        <f>_xlfn.STDEV.S(S4:S9)</f>
-        <v>1.4288690166235207</v>
-      </c>
-      <c r="AA4">
-        <f>AVERAGE(T4:T9)</f>
-        <v>20.583333333333332</v>
-      </c>
-      <c r="AB4">
-        <f>_xlfn.STDEV.S(T4:T9)</f>
-        <v>1.0368220676663862</v>
-      </c>
-      <c r="AC4">
-        <f>MIN(Q4:S4)</f>
-        <v>12.5</v>
-      </c>
-      <c r="AD4">
-        <f>(T4-AC4)</f>
-        <v>7.8333333333333321</v>
-      </c>
-      <c r="AE4">
-        <f>AVERAGE(AD4:AD9)</f>
-        <v>5.666666666666667</v>
-      </c>
-      <c r="AF4">
-        <f>_xlfn.STDEV.S(AD4:AD9)</f>
-        <v>1.7224014243685055</v>
-      </c>
-    </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B5">
-        <v>88</v>
-      </c>
-      <c r="C5">
-        <v>12</v>
-      </c>
-      <c r="D5">
-        <v>20</v>
-      </c>
-      <c r="E5">
-        <v>80</v>
-      </c>
-      <c r="G5">
-        <v>71</v>
-      </c>
-      <c r="H5">
-        <v>29</v>
-      </c>
-      <c r="I5">
-        <v>5</v>
-      </c>
-      <c r="J5">
-        <v>95</v>
-      </c>
-      <c r="L5">
-        <v>67</v>
-      </c>
-      <c r="M5">
-        <v>33</v>
-      </c>
-      <c r="N5">
-        <v>18</v>
-      </c>
-      <c r="O5">
-        <v>82</v>
-      </c>
-      <c r="Q5">
-        <f t="shared" ref="Q5:Q9" si="0">AVERAGE(C5,D5)</f>
-        <v>16</v>
-      </c>
-      <c r="R5">
-        <f t="shared" ref="R5:R9" si="1">AVERAGE(H5,I5)</f>
-        <v>17</v>
-      </c>
-      <c r="S5">
-        <f t="shared" ref="S5:S9" si="2">AVERAGE(M5,N5)</f>
-        <v>25.5</v>
-      </c>
-      <c r="T5">
-        <f t="shared" ref="T5:T9" si="3">AVERAGE(Q5:S5)</f>
-        <v>19.5</v>
-      </c>
-      <c r="AC5">
-        <f t="shared" ref="AC5:AC9" si="4">MIN(Q5:S5)</f>
-        <v>16</v>
-      </c>
-      <c r="AD5">
-        <f t="shared" ref="AD5:AD9" si="5">(T5-AC5)</f>
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B6">
-        <v>92</v>
-      </c>
-      <c r="C6">
-        <v>8</v>
-      </c>
-      <c r="D6">
-        <v>21</v>
-      </c>
-      <c r="E6">
-        <v>79</v>
-      </c>
-      <c r="G6">
-        <v>78</v>
-      </c>
-      <c r="H6">
-        <v>22</v>
-      </c>
-      <c r="I6">
-        <v>15</v>
-      </c>
-      <c r="J6">
-        <v>85</v>
-      </c>
-      <c r="L6">
-        <v>62</v>
-      </c>
-      <c r="M6">
-        <v>38</v>
-      </c>
-      <c r="N6">
-        <v>18</v>
-      </c>
-      <c r="O6">
-        <v>82</v>
-      </c>
-      <c r="Q6">
-        <f t="shared" si="0"/>
-        <v>14.5</v>
-      </c>
-      <c r="R6">
-        <f t="shared" si="1"/>
-        <v>18.5</v>
-      </c>
-      <c r="S6">
-        <f t="shared" si="2"/>
-        <v>28</v>
-      </c>
-      <c r="T6">
-        <f t="shared" si="3"/>
-        <v>20.333333333333332</v>
-      </c>
-      <c r="AC6">
-        <f t="shared" si="4"/>
-        <v>14.5</v>
-      </c>
-      <c r="AD6">
-        <f t="shared" si="5"/>
-        <v>5.8333333333333321</v>
-      </c>
-    </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B7">
-        <v>81</v>
-      </c>
-      <c r="C7">
-        <v>19</v>
-      </c>
-      <c r="D7">
-        <v>13</v>
-      </c>
-      <c r="E7">
-        <v>87</v>
-      </c>
-      <c r="G7">
-        <v>65</v>
-      </c>
-      <c r="H7">
-        <v>35</v>
-      </c>
-      <c r="I7">
-        <v>7</v>
-      </c>
-      <c r="J7">
-        <v>93</v>
-      </c>
-      <c r="L7">
-        <v>67</v>
-      </c>
-      <c r="M7">
-        <v>33</v>
-      </c>
-      <c r="N7">
-        <v>18</v>
-      </c>
-      <c r="O7">
-        <v>82</v>
-      </c>
-      <c r="Q7">
-        <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="R7">
-        <f t="shared" si="1"/>
-        <v>21</v>
-      </c>
-      <c r="S7">
-        <f t="shared" si="2"/>
-        <v>25.5</v>
-      </c>
-      <c r="T7">
-        <f t="shared" si="3"/>
-        <v>20.833333333333332</v>
-      </c>
-      <c r="AC7">
-        <f t="shared" si="4"/>
-        <v>16</v>
-      </c>
-      <c r="AD7">
-        <f t="shared" si="5"/>
-        <v>4.8333333333333321</v>
-      </c>
-    </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B8">
-        <v>80</v>
-      </c>
-      <c r="C8">
-        <v>20</v>
-      </c>
-      <c r="D8">
-        <v>16</v>
-      </c>
-      <c r="E8">
-        <v>84</v>
-      </c>
-      <c r="G8">
-        <v>60</v>
-      </c>
-      <c r="H8">
-        <v>40</v>
-      </c>
-      <c r="I8">
-        <v>8</v>
-      </c>
-      <c r="J8">
-        <v>92</v>
-      </c>
-      <c r="L8">
-        <v>66</v>
-      </c>
-      <c r="M8">
-        <v>34</v>
-      </c>
-      <c r="N8">
-        <v>17</v>
-      </c>
-      <c r="O8">
-        <v>83</v>
-      </c>
-      <c r="Q8">
-        <f t="shared" si="0"/>
-        <v>18</v>
-      </c>
-      <c r="R8">
-        <f t="shared" si="1"/>
-        <v>24</v>
-      </c>
-      <c r="S8">
-        <f t="shared" si="2"/>
-        <v>25.5</v>
-      </c>
-      <c r="T8">
-        <f t="shared" si="3"/>
-        <v>22.5</v>
-      </c>
-      <c r="AC8">
-        <f t="shared" si="4"/>
-        <v>18</v>
-      </c>
-      <c r="AD8">
-        <f t="shared" si="5"/>
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B9">
-        <v>91</v>
-      </c>
-      <c r="C9">
-        <v>9</v>
-      </c>
-      <c r="D9">
-        <v>16</v>
-      </c>
-      <c r="E9">
-        <v>84</v>
-      </c>
-      <c r="G9">
-        <v>66</v>
-      </c>
-      <c r="H9">
-        <v>34</v>
-      </c>
-      <c r="I9">
-        <v>10</v>
-      </c>
-      <c r="J9">
-        <v>90</v>
-      </c>
-      <c r="L9">
-        <v>68</v>
-      </c>
-      <c r="M9">
-        <v>32</v>
-      </c>
-      <c r="N9">
-        <v>19</v>
-      </c>
-      <c r="O9">
-        <v>81</v>
-      </c>
-      <c r="Q9">
-        <f t="shared" si="0"/>
-        <v>12.5</v>
-      </c>
-      <c r="R9">
-        <f t="shared" si="1"/>
-        <v>22</v>
-      </c>
-      <c r="S9">
-        <f t="shared" si="2"/>
-        <v>25.5</v>
-      </c>
-      <c r="T9">
-        <f t="shared" si="3"/>
-        <v>20</v>
-      </c>
-      <c r="AC9">
-        <f t="shared" si="4"/>
-        <v>12.5</v>
-      </c>
-      <c r="AD9">
-        <f t="shared" si="5"/>
-        <v>7.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="11" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B11">
-        <v>86</v>
-      </c>
-      <c r="C11">
-        <v>14</v>
-      </c>
-      <c r="D11">
-        <v>20</v>
-      </c>
-      <c r="E11">
-        <v>80</v>
-      </c>
-      <c r="G11">
-        <v>75</v>
-      </c>
-      <c r="H11">
-        <v>25</v>
-      </c>
-      <c r="I11">
-        <v>8</v>
-      </c>
-      <c r="J11">
-        <v>92</v>
-      </c>
-      <c r="L11">
-        <v>67</v>
-      </c>
-      <c r="M11">
-        <v>33</v>
-      </c>
-      <c r="N11">
-        <v>27</v>
-      </c>
-      <c r="O11">
-        <v>73</v>
-      </c>
-      <c r="Q11">
-        <f t="shared" ref="Q11:Q14" si="6">AVERAGE(C11,D11)</f>
-        <v>17</v>
-      </c>
-      <c r="R11">
-        <f t="shared" ref="R11:R14" si="7">AVERAGE(H11,I11)</f>
-        <v>16.5</v>
-      </c>
-      <c r="S11">
-        <f t="shared" ref="S11:S14" si="8">AVERAGE(M11,N11)</f>
-        <v>30</v>
-      </c>
-      <c r="T11">
-        <f t="shared" ref="T11:T14" si="9">AVERAGE(Q11:S11)</f>
-        <v>21.166666666666668</v>
-      </c>
-      <c r="U11">
-        <f>AVERAGE(Q11:Q16)</f>
-        <v>16.5</v>
-      </c>
-      <c r="V11">
-        <f>_xlfn.STDEV.S(Q11:Q16)</f>
-        <v>0.70710678118654757</v>
-      </c>
-      <c r="W11">
-        <f>AVERAGE(R11:R16)</f>
-        <v>17.25</v>
-      </c>
-      <c r="X11">
-        <f>_xlfn.STDEV.S(R11:R16)</f>
-        <v>3.378855822118882</v>
-      </c>
-      <c r="Y11">
-        <f>AVERAGE(S11:S16)</f>
-        <v>31.25</v>
-      </c>
-      <c r="Z11">
-        <f>_xlfn.STDEV.S(S11:S16)</f>
-        <v>3.1754264805429417</v>
-      </c>
-      <c r="AA11">
-        <f>AVERAGE(T11:T16)</f>
-        <v>21.666666666666668</v>
-      </c>
-      <c r="AB11">
-        <f>_xlfn.STDEV.S(T11:T16)</f>
-        <v>2.2730302828309759</v>
-      </c>
-      <c r="AC11">
-        <f t="shared" ref="AC11:AC14" si="10">MIN(Q11:S11)</f>
-        <v>16.5</v>
-      </c>
-      <c r="AD11">
-        <f t="shared" ref="AD11:AD14" si="11">(T11-AC11)</f>
-        <v>4.6666666666666679</v>
-      </c>
-      <c r="AE11">
-        <f>AVERAGE(AD11:AD16)</f>
-        <v>5.7916666666666679</v>
-      </c>
-      <c r="AF11">
-        <f>_xlfn.STDEV.S(AD11:AD16)</f>
-        <v>1.6007810593582092</v>
-      </c>
-    </row>
-    <row r="12" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B12">
-        <v>95</v>
-      </c>
-      <c r="C12">
-        <v>5</v>
-      </c>
-      <c r="D12">
-        <v>28</v>
-      </c>
-      <c r="E12">
-        <v>72</v>
-      </c>
-      <c r="G12">
-        <v>67</v>
-      </c>
-      <c r="H12">
-        <v>33</v>
-      </c>
-      <c r="I12">
-        <v>11</v>
-      </c>
-      <c r="J12">
-        <v>89</v>
-      </c>
-      <c r="L12">
-        <v>65</v>
-      </c>
-      <c r="M12">
-        <v>35</v>
-      </c>
-      <c r="N12">
-        <v>36</v>
-      </c>
-      <c r="O12">
-        <v>64</v>
-      </c>
-      <c r="Q12">
-        <f t="shared" si="6"/>
-        <v>16.5</v>
-      </c>
-      <c r="R12">
-        <f t="shared" si="7"/>
-        <v>22</v>
-      </c>
-      <c r="S12">
-        <f t="shared" si="8"/>
-        <v>35.5</v>
-      </c>
-      <c r="T12">
-        <f t="shared" si="9"/>
-        <v>24.666666666666668</v>
-      </c>
-      <c r="AC12">
-        <f t="shared" si="10"/>
-        <v>16.5</v>
-      </c>
-      <c r="AD12">
-        <f t="shared" si="11"/>
-        <v>8.1666666666666679</v>
-      </c>
-    </row>
-    <row r="13" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B13">
-        <v>87</v>
-      </c>
-      <c r="C13">
-        <v>13</v>
-      </c>
-      <c r="D13">
-        <v>18</v>
-      </c>
-      <c r="E13">
-        <v>82</v>
-      </c>
-      <c r="G13">
-        <v>76</v>
-      </c>
-      <c r="H13">
-        <v>24</v>
-      </c>
-      <c r="I13">
-        <v>4</v>
-      </c>
-      <c r="J13">
-        <v>96</v>
-      </c>
-      <c r="L13">
-        <v>70</v>
-      </c>
-      <c r="M13">
-        <v>30</v>
-      </c>
-      <c r="N13">
-        <v>26</v>
-      </c>
-      <c r="O13">
-        <v>74</v>
-      </c>
-      <c r="Q13">
-        <f t="shared" si="6"/>
-        <v>15.5</v>
-      </c>
-      <c r="R13">
-        <f t="shared" si="7"/>
-        <v>14</v>
-      </c>
-      <c r="S13">
-        <f t="shared" si="8"/>
-        <v>28</v>
-      </c>
-      <c r="T13">
-        <f t="shared" si="9"/>
-        <v>19.166666666666668</v>
-      </c>
-      <c r="AC13">
-        <f t="shared" si="10"/>
-        <v>14</v>
-      </c>
-      <c r="AD13">
-        <f t="shared" si="11"/>
-        <v>5.1666666666666679</v>
-      </c>
-    </row>
-    <row r="14" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="B14">
-        <v>80</v>
-      </c>
-      <c r="C14">
-        <v>20</v>
-      </c>
-      <c r="D14">
-        <v>14</v>
-      </c>
-      <c r="E14">
-        <v>86</v>
-      </c>
-      <c r="G14">
-        <v>71</v>
-      </c>
-      <c r="H14">
-        <v>29</v>
-      </c>
-      <c r="I14">
-        <v>4</v>
-      </c>
-      <c r="J14">
-        <v>96</v>
-      </c>
-      <c r="L14">
-        <v>62</v>
-      </c>
-      <c r="M14">
-        <v>38</v>
-      </c>
-      <c r="N14">
-        <v>25</v>
-      </c>
-      <c r="O14">
-        <v>75</v>
-      </c>
-      <c r="Q14">
-        <f t="shared" si="6"/>
-        <v>17</v>
-      </c>
-      <c r="R14">
-        <f t="shared" si="7"/>
-        <v>16.5</v>
-      </c>
-      <c r="S14">
-        <f t="shared" si="8"/>
-        <v>31.5</v>
-      </c>
-      <c r="T14">
-        <f t="shared" si="9"/>
-        <v>21.666666666666668</v>
-      </c>
-      <c r="AC14">
-        <f t="shared" si="10"/>
-        <v>16.5</v>
-      </c>
-      <c r="AD14">
-        <f t="shared" si="11"/>
-        <v>5.1666666666666679</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>